<commit_message>
auto stock scan 2026-10-12 17:13 UTC
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N38"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="L3" s="11" t="n">
-        <v>97.3</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="M3" s="8" t="inlineStr">
         <is>
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="L4" s="4" t="n">
-        <v>94.59999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="M4" s="8" t="inlineStr">
         <is>
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="L5" s="11" t="n">
-        <v>91.90000000000001</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="M5" s="8" t="inlineStr">
         <is>
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>89.2</v>
+        <v>89.5</v>
       </c>
       <c r="M6" s="8" t="inlineStr">
         <is>
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="L7" s="11" t="n">
-        <v>82.40000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="M7" s="8" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>82.40000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="M8" s="8" t="inlineStr">
         <is>
@@ -1131,7 +1131,7 @@
         </is>
       </c>
       <c r="L9" s="11" t="n">
-        <v>82.40000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="M9" s="8" t="inlineStr">
         <is>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="L10" s="4" t="n">
-        <v>82.40000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="M10" s="8" t="inlineStr">
         <is>
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="L11" s="11" t="n">
-        <v>75.7</v>
+        <v>76.3</v>
       </c>
       <c r="M11" s="8" t="inlineStr">
         <is>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="L12" s="4" t="n">
-        <v>71.59999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="M12" s="8" t="inlineStr">
         <is>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="L13" s="11" t="n">
-        <v>71.59999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="M13" s="8" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
         </is>
       </c>
       <c r="L14" s="4" t="n">
-        <v>64.90000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="M14" s="8" t="inlineStr">
         <is>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="L15" s="11" t="n">
-        <v>64.90000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="M15" s="8" t="inlineStr">
         <is>
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="L16" s="4" t="n">
-        <v>64.90000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="M16" s="8" t="inlineStr">
         <is>
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="L17" s="11" t="n">
-        <v>59.5</v>
+        <v>60.5</v>
       </c>
       <c r="M17" s="8" t="inlineStr">
         <is>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="L18" s="4" t="n">
-        <v>56.8</v>
+        <v>57.9</v>
       </c>
       <c r="M18" s="8" t="inlineStr">
         <is>
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="L19" s="11" t="n">
-        <v>51.4</v>
+        <v>52.6</v>
       </c>
       <c r="M19" s="8" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         </is>
       </c>
       <c r="L20" s="4" t="n">
-        <v>51.4</v>
+        <v>52.6</v>
       </c>
       <c r="M20" s="8" t="inlineStr">
         <is>
@@ -1831,7 +1831,7 @@
         </is>
       </c>
       <c r="L21" s="11" t="n">
-        <v>51.4</v>
+        <v>52.6</v>
       </c>
       <c r="M21" s="8" t="inlineStr">
         <is>
@@ -1895,7 +1895,7 @@
         </is>
       </c>
       <c r="L22" s="4" t="n">
-        <v>44.6</v>
+        <v>46.1</v>
       </c>
       <c r="M22" s="8" t="inlineStr">
         <is>
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="L23" s="11" t="n">
-        <v>44.6</v>
+        <v>46.1</v>
       </c>
       <c r="M23" s="8" t="inlineStr">
         <is>
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="L24" s="4" t="n">
-        <v>37.8</v>
+        <v>39.5</v>
       </c>
       <c r="M24" s="8" t="inlineStr">
         <is>
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="L25" s="11" t="n">
-        <v>37.8</v>
+        <v>39.5</v>
       </c>
       <c r="M25" s="8" t="inlineStr">
         <is>
@@ -2123,7 +2123,7 @@
         </is>
       </c>
       <c r="L26" s="4" t="n">
-        <v>37.8</v>
+        <v>39.5</v>
       </c>
       <c r="M26" s="8" t="inlineStr">
         <is>
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="L27" s="11" t="n">
-        <v>31.1</v>
+        <v>32.9</v>
       </c>
       <c r="M27" s="8" t="inlineStr">
         <is>
@@ -2235,7 +2235,7 @@
         </is>
       </c>
       <c r="L28" s="4" t="n">
-        <v>31.1</v>
+        <v>32.9</v>
       </c>
       <c r="M28" s="8" t="inlineStr">
         <is>
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="L29" s="11" t="n">
-        <v>27</v>
+        <v>28.9</v>
       </c>
       <c r="M29" s="8" t="inlineStr">
         <is>
@@ -2307,19 +2307,19 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SZ002240</t>
+          <t>SZ300831</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>盛新锂能</t>
+          <t>派瑞股份</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>23.58</v>
+        <v>12.85</v>
       </c>
       <c r="D30" s="14" t="n">
-        <v>-6.98</v>
+        <v>-1</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>20</v>
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="L30" s="4" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="M30" s="8" t="inlineStr">
         <is>
@@ -2363,19 +2363,19 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>SZ000919</t>
+          <t>SZ002240</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>金陵药业</t>
+          <t>盛新锂能</t>
         </is>
       </c>
       <c r="C31" s="11" t="n">
-        <v>6.53</v>
+        <v>23.58</v>
       </c>
       <c r="D31" s="16" t="n">
-        <v>-2.1</v>
+        <v>-6.98</v>
       </c>
       <c r="E31" s="9" t="n">
         <v>20</v>
@@ -2390,11 +2390,7 @@
           <t>排除/止损 | 弱市慎加仓</t>
         </is>
       </c>
-      <c r="H31" s="9" t="inlineStr">
-        <is>
-          <t>MACD金叉</t>
-        </is>
-      </c>
+      <c r="H31" s="9" t="inlineStr"/>
       <c r="I31" s="9" t="inlineStr"/>
       <c r="J31" s="9" t="inlineStr">
         <is>
@@ -2403,11 +2399,11 @@
       </c>
       <c r="K31" s="7" t="inlineStr">
         <is>
-          <t>弱市</t>
+          <t>深回撤|弱市</t>
         </is>
       </c>
       <c r="L31" s="11" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="M31" s="8" t="inlineStr">
         <is>
@@ -2423,19 +2419,19 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>SZ002402</t>
+          <t>SZ000919</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>和而泰</t>
+          <t>金陵药业</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>17.21</v>
+        <v>6.53</v>
       </c>
       <c r="D32" s="14" t="n">
-        <v>-1.88</v>
+        <v>-2.1</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>20</v>
@@ -2450,7 +2446,11 @@
           <t>排除/止损 | 弱市慎加仓</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>MACD金叉</t>
+        </is>
+      </c>
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
@@ -2459,11 +2459,11 @@
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>深回撤|弱市</t>
+          <t>弱市</t>
         </is>
       </c>
       <c r="L32" s="4" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="M32" s="8" t="inlineStr">
         <is>
@@ -2479,19 +2479,19 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>SZ002475</t>
+          <t>SZ002402</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>立讯精密</t>
+          <t>和而泰</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>46.32</v>
+        <v>17.21</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>-2.67</v>
+        <v>-1.88</v>
       </c>
       <c r="E33" s="9" t="n">
         <v>20</v>
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="L33" s="11" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="M33" s="8" t="inlineStr">
         <is>
@@ -2535,19 +2535,19 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SZ002241</t>
+          <t>SZ002475</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>歌尔股份</t>
+          <t>立讯精密</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>20.85</v>
+        <v>46.32</v>
       </c>
       <c r="D34" s="14" t="n">
-        <v>-3.07</v>
+        <v>-2.67</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>20</v>
@@ -2571,11 +2571,11 @@
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>弱市</t>
+          <t>深回撤|弱市</t>
         </is>
       </c>
       <c r="L34" s="4" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="M34" s="8" t="inlineStr">
         <is>
@@ -2591,19 +2591,19 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>SZ300442</t>
+          <t>SZ002241</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>润泽科技</t>
+          <t>歌尔股份</t>
         </is>
       </c>
       <c r="C35" s="11" t="n">
-        <v>57.64</v>
+        <v>20.85</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>-1.69</v>
+        <v>-3.07</v>
       </c>
       <c r="E35" s="9" t="n">
         <v>20</v>
@@ -2627,11 +2627,11 @@
       </c>
       <c r="K35" s="7" t="inlineStr">
         <is>
-          <t>深回撤|弱市</t>
+          <t>弱市</t>
         </is>
       </c>
       <c r="L35" s="11" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="M35" s="8" t="inlineStr">
         <is>
@@ -2647,22 +2647,22 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>SZ002202</t>
+          <t>SZ300442</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>金风科技</t>
+          <t>润泽科技</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>16.06</v>
+        <v>57.64</v>
       </c>
       <c r="D36" s="14" t="n">
-        <v>-1.77</v>
+        <v>-1.69</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F36" s="18" t="inlineStr">
         <is>
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="L36" s="4" t="n">
-        <v>8.1</v>
+        <v>18.4</v>
       </c>
       <c r="M36" s="8" t="inlineStr">
         <is>
@@ -2703,22 +2703,22 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>SZ002245</t>
+          <t>SZ002202</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>蔚蓝锂芯</t>
+          <t>金风科技</t>
         </is>
       </c>
       <c r="C37" s="11" t="n">
-        <v>15.77</v>
+        <v>16.06</v>
       </c>
       <c r="D37" s="16" t="n">
-        <v>-1.99</v>
+        <v>-1.77</v>
       </c>
       <c r="E37" s="9" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F37" s="18" t="inlineStr">
         <is>
@@ -2743,7 +2743,7 @@
         </is>
       </c>
       <c r="L37" s="11" t="n">
-        <v>4.1</v>
+        <v>7.9</v>
       </c>
       <c r="M37" s="8" t="inlineStr">
         <is>
@@ -2759,19 +2759,19 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>SZ000657</t>
+          <t>SZ002245</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>中钨高新</t>
+          <t>蔚蓝锂芯</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>48.34</v>
+        <v>15.77</v>
       </c>
       <c r="D38" s="14" t="n">
-        <v>-5.46</v>
+        <v>-1.99</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>10</v>
@@ -2799,7 +2799,7 @@
         </is>
       </c>
       <c r="L38" s="4" t="n">
-        <v>4.1</v>
+        <v>3.9</v>
       </c>
       <c r="M38" s="8" t="inlineStr">
         <is>
@@ -2807,13 +2807,69 @@
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>SZ000657</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>中钨高新</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="n">
+        <v>48.34</v>
+      </c>
+      <c r="D39" s="16" t="n">
+        <v>-5.46</v>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F39" s="18" t="inlineStr">
+        <is>
+          <t>D 级 (风险)</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>排除/止损 | 弱市慎加仓</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr"/>
+      <c r="I39" s="9" t="inlineStr"/>
+      <c r="J39" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>深回撤|弱市</t>
+        </is>
+      </c>
+      <c r="L39" s="11" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="M39" s="8" t="inlineStr">
+        <is>
+          <t>弱势</t>
+        </is>
+      </c>
+      <c r="N39" s="9" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E38">
+  <conditionalFormatting sqref="E2:E39">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="15"/>
@@ -2825,7 +2881,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L38">
+  <conditionalFormatting sqref="L2:L39">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -3186,40 +3242,40 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
+        <v>24271.2</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>24211.35</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>23785.79</v>
-      </c>
       <c r="E4" s="4" t="n">
-        <v>23941.26</v>
+        <v>24434.93</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>24224.05</v>
+        <v>24455.95</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>23941.26</v>
+        <v>24193.3</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>1.79</v>
+        <v>0.25</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1.19</v>
+        <v>1.08</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>24089.708</v>
+        <v>24135.88</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>24271.027</v>
+        <v>24247.138</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>24817.064</v>
+        <v>24773.278</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>25156.338</v>
+        <v>25151.488</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>25079.441</v>
+        <v>25062.025</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>23737.14</v>
@@ -3231,7 +3287,7 @@
         <v>23737.14</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>24354.11</v>
+        <v>24455.95</v>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
@@ -3240,12 +3296,12 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>无明显形态</t>
+          <t>近期连阳</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>光脚大阳</t>
+          <t>小阴线</t>
         </is>
       </c>
       <c r="V4" s="2" t="n">
@@ -3258,7 +3314,7 @@
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>跌破MA60 | 日内偏强</t>
+          <t>跌破MA60 | 近期连阳</t>
         </is>
       </c>
     </row>
@@ -3273,7 +3329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ38"/>
+  <dimension ref="A1:CQ39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4185,7 +4241,7 @@
         <v>100</v>
       </c>
       <c r="CP2" s="4" t="n">
-        <v>97.3</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="CQ2" s="2" t="inlineStr">
         <is>
@@ -4517,10 +4573,10 @@
         </is>
       </c>
       <c r="CO3" s="11" t="n">
-        <v>97.3</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="CP3" s="11" t="n">
-        <v>94.59999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="CQ3" s="9" t="inlineStr">
         <is>
@@ -4852,7 +4908,7 @@
         </is>
       </c>
       <c r="CO4" s="4" t="n">
-        <v>94.59999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="CP4" s="4" t="n">
         <v>100</v>
@@ -5187,10 +5243,10 @@
         </is>
       </c>
       <c r="CO5" s="11" t="n">
-        <v>91.90000000000001</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="CP5" s="11" t="n">
-        <v>91.90000000000001</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="CQ5" s="9" t="inlineStr">
         <is>
@@ -5522,10 +5578,10 @@
         </is>
       </c>
       <c r="CO6" s="4" t="n">
-        <v>89.2</v>
+        <v>89.5</v>
       </c>
       <c r="CP6" s="4" t="n">
-        <v>78.40000000000001</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="CQ6" s="2" t="inlineStr">
         <is>
@@ -5857,10 +5913,10 @@
         </is>
       </c>
       <c r="CO7" s="11" t="n">
-        <v>82.40000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="CP7" s="11" t="n">
-        <v>67.59999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="CQ7" s="9" t="inlineStr">
         <is>
@@ -6192,10 +6248,10 @@
         </is>
       </c>
       <c r="CO8" s="4" t="n">
-        <v>82.40000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="CP8" s="4" t="n">
-        <v>62.2</v>
+        <v>63.2</v>
       </c>
       <c r="CQ8" s="2" t="inlineStr">
         <is>
@@ -6535,10 +6591,10 @@
         </is>
       </c>
       <c r="CO9" s="11" t="n">
-        <v>82.40000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="CP9" s="11" t="n">
-        <v>81.09999999999999</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="CQ9" s="9" t="inlineStr">
         <is>
@@ -6874,10 +6930,10 @@
         </is>
       </c>
       <c r="CO10" s="4" t="n">
-        <v>82.40000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="CP10" s="4" t="n">
-        <v>51.4</v>
+        <v>52.6</v>
       </c>
       <c r="CQ10" s="2" t="inlineStr">
         <is>
@@ -7213,10 +7269,10 @@
         </is>
       </c>
       <c r="CO11" s="11" t="n">
-        <v>75.7</v>
+        <v>76.3</v>
       </c>
       <c r="CP11" s="11" t="n">
-        <v>83.8</v>
+        <v>84.2</v>
       </c>
       <c r="CQ11" s="9" t="inlineStr">
         <is>
@@ -7548,10 +7604,10 @@
         </is>
       </c>
       <c r="CO12" s="4" t="n">
-        <v>71.59999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="CP12" s="4" t="n">
-        <v>75.7</v>
+        <v>76.3</v>
       </c>
       <c r="CQ12" s="2" t="inlineStr">
         <is>
@@ -7883,10 +7939,10 @@
         </is>
       </c>
       <c r="CO13" s="11" t="n">
-        <v>71.59999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="CP13" s="11" t="n">
-        <v>59.5</v>
+        <v>60.5</v>
       </c>
       <c r="CQ13" s="9" t="inlineStr">
         <is>
@@ -8222,10 +8278,10 @@
         </is>
       </c>
       <c r="CO14" s="4" t="n">
-        <v>64.90000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="CP14" s="4" t="n">
-        <v>43.2</v>
+        <v>44.7</v>
       </c>
       <c r="CQ14" s="2" t="inlineStr">
         <is>
@@ -8277,7 +8333,7 @@
         <v>1.25</v>
       </c>
       <c r="M15" s="11" t="n">
-        <v>3.09</v>
+        <v>0.03</v>
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
@@ -8288,7 +8344,7 @@
         <v>1.25</v>
       </c>
       <c r="P15" s="11" t="n">
-        <v>11.64</v>
+        <v>0.12</v>
       </c>
       <c r="Q15" s="11" t="n">
         <v>0</v>
@@ -8357,7 +8413,7 @@
         <v>5.52</v>
       </c>
       <c r="AK15" s="11" t="n">
-        <v>11.5</v>
+        <v>11.46</v>
       </c>
       <c r="AL15" s="8" t="inlineStr">
         <is>
@@ -8439,7 +8495,7 @@
         <v>56.65</v>
       </c>
       <c r="BG15" s="11" t="n">
-        <v>63.76</v>
+        <v>63.75</v>
       </c>
       <c r="BH15" s="20" t="inlineStr">
         <is>
@@ -8447,7 +8503,7 @@
         </is>
       </c>
       <c r="BI15" s="11" t="n">
-        <v>-9.550000000000001</v>
+        <v>-9.69</v>
       </c>
       <c r="BJ15" s="11" t="n">
         <v>19.6</v>
@@ -8482,7 +8538,7 @@
         <v>26.029</v>
       </c>
       <c r="BT15" s="11" t="n">
-        <v>26.328</v>
+        <v>26.337</v>
       </c>
       <c r="BU15" s="11" t="n">
         <v>0</v>
@@ -8512,7 +8568,7 @@
         </is>
       </c>
       <c r="CB15" s="11" t="n">
-        <v>1.3</v>
+        <v>1.26</v>
       </c>
       <c r="CC15" s="20" t="inlineStr">
         <is>
@@ -8557,10 +8613,10 @@
         </is>
       </c>
       <c r="CO15" s="11" t="n">
-        <v>64.90000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="CP15" s="11" t="n">
-        <v>64.90000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="CQ15" s="9" t="inlineStr">
         <is>
@@ -8896,10 +8952,10 @@
         </is>
       </c>
       <c r="CO16" s="4" t="n">
-        <v>64.90000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="CP16" s="4" t="n">
-        <v>70.3</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="CQ16" s="2" t="inlineStr">
         <is>
@@ -9235,10 +9291,10 @@
         </is>
       </c>
       <c r="CO17" s="11" t="n">
-        <v>59.5</v>
+        <v>60.5</v>
       </c>
       <c r="CP17" s="11" t="n">
-        <v>89.2</v>
+        <v>89.5</v>
       </c>
       <c r="CQ17" s="9" t="inlineStr">
         <is>
@@ -9570,10 +9626,10 @@
         </is>
       </c>
       <c r="CO18" s="4" t="n">
-        <v>56.8</v>
+        <v>57.9</v>
       </c>
       <c r="CP18" s="4" t="n">
-        <v>86.5</v>
+        <v>86.8</v>
       </c>
       <c r="CQ18" s="2" t="inlineStr">
         <is>
@@ -9905,10 +9961,10 @@
         </is>
       </c>
       <c r="CO19" s="11" t="n">
-        <v>51.4</v>
+        <v>52.6</v>
       </c>
       <c r="CP19" s="11" t="n">
-        <v>35.1</v>
+        <v>36.8</v>
       </c>
       <c r="CQ19" s="9" t="inlineStr">
         <is>
@@ -10244,10 +10300,10 @@
         </is>
       </c>
       <c r="CO20" s="4" t="n">
-        <v>51.4</v>
+        <v>52.6</v>
       </c>
       <c r="CP20" s="4" t="n">
-        <v>40.5</v>
+        <v>42.1</v>
       </c>
       <c r="CQ20" s="2" t="inlineStr">
         <is>
@@ -10583,10 +10639,10 @@
         </is>
       </c>
       <c r="CO21" s="11" t="n">
-        <v>51.4</v>
+        <v>52.6</v>
       </c>
       <c r="CP21" s="11" t="n">
-        <v>48.6</v>
+        <v>50</v>
       </c>
       <c r="CQ21" s="9" t="inlineStr">
         <is>
@@ -10926,10 +10982,10 @@
         </is>
       </c>
       <c r="CO22" s="4" t="n">
-        <v>44.6</v>
+        <v>46.1</v>
       </c>
       <c r="CP22" s="4" t="n">
-        <v>18.9</v>
+        <v>18.4</v>
       </c>
       <c r="CQ22" s="2" t="inlineStr">
         <is>
@@ -11261,10 +11317,10 @@
         </is>
       </c>
       <c r="CO23" s="11" t="n">
-        <v>44.6</v>
+        <v>46.1</v>
       </c>
       <c r="CP23" s="11" t="n">
-        <v>21.6</v>
+        <v>21.1</v>
       </c>
       <c r="CQ23" s="9" t="inlineStr">
         <is>
@@ -11596,10 +11652,10 @@
         </is>
       </c>
       <c r="CO24" s="4" t="n">
-        <v>37.8</v>
+        <v>39.5</v>
       </c>
       <c r="CP24" s="4" t="n">
-        <v>54.1</v>
+        <v>55.3</v>
       </c>
       <c r="CQ24" s="2" t="inlineStr">
         <is>
@@ -11935,10 +11991,10 @@
         </is>
       </c>
       <c r="CO25" s="11" t="n">
-        <v>37.8</v>
+        <v>39.5</v>
       </c>
       <c r="CP25" s="11" t="n">
-        <v>32.4</v>
+        <v>34.2</v>
       </c>
       <c r="CQ25" s="9" t="inlineStr">
         <is>
@@ -12270,10 +12326,10 @@
         </is>
       </c>
       <c r="CO26" s="4" t="n">
-        <v>37.8</v>
+        <v>39.5</v>
       </c>
       <c r="CP26" s="4" t="n">
-        <v>8.1</v>
+        <v>7.9</v>
       </c>
       <c r="CQ26" s="2" t="inlineStr">
         <is>
@@ -12605,10 +12661,10 @@
         </is>
       </c>
       <c r="CO27" s="11" t="n">
-        <v>31.1</v>
+        <v>32.9</v>
       </c>
       <c r="CP27" s="11" t="n">
-        <v>45.9</v>
+        <v>47.4</v>
       </c>
       <c r="CQ27" s="9" t="inlineStr">
         <is>
@@ -12940,10 +12996,10 @@
         </is>
       </c>
       <c r="CO28" s="4" t="n">
-        <v>31.1</v>
+        <v>32.9</v>
       </c>
       <c r="CP28" s="4" t="n">
-        <v>10.8</v>
+        <v>10.5</v>
       </c>
       <c r="CQ28" s="2" t="inlineStr">
         <is>
@@ -13275,10 +13331,10 @@
         </is>
       </c>
       <c r="CO29" s="11" t="n">
-        <v>27</v>
+        <v>28.9</v>
       </c>
       <c r="CP29" s="11" t="n">
-        <v>24.3</v>
+        <v>23.7</v>
       </c>
       <c r="CQ29" s="9" t="inlineStr">
         <is>
@@ -13289,16 +13345,16 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SZ002240</t>
+          <t>SZ300831</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>盛新锂能</t>
+          <t>派瑞股份</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>23.58</v>
+        <v>12.85</v>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
@@ -13306,31 +13362,31 @@
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>25.35</v>
+        <v>12.98</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>24.5</v>
+        <v>12.88</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>25.09</v>
+        <v>13.17</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>23.52</v>
+        <v>12.72</v>
       </c>
       <c r="I30" s="4" t="n">
-        <v>24.06</v>
+        <v>12.91</v>
       </c>
       <c r="J30" s="14" t="n">
-        <v>-6.98</v>
+        <v>-1</v>
       </c>
       <c r="K30" s="4" t="n">
-        <v>6.19</v>
+        <v>3.47</v>
       </c>
       <c r="L30" s="4" t="n">
-        <v>1.35</v>
+        <v>1.03</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>7.9</v>
+        <v>0</v>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
@@ -13338,10 +13394,10 @@
         </is>
       </c>
       <c r="O30" s="4" t="n">
-        <v>3.58</v>
+        <v>1.57</v>
       </c>
       <c r="P30" s="4" t="n">
-        <v>32.65</v>
+        <v>0.03</v>
       </c>
       <c r="Q30" s="4" t="n">
         <v>0</v>
@@ -13356,37 +13412,37 @@
         <v>0</v>
       </c>
       <c r="U30" s="14" t="n">
-        <v>-6.21</v>
+        <v>-2.21</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>5.53</v>
+        <v>3.79</v>
       </c>
       <c r="W30" s="4" t="n">
-        <v>24.69</v>
+        <v>12.99</v>
       </c>
       <c r="X30" s="4" t="n">
-        <v>24.5</v>
+        <v>12.88</v>
       </c>
       <c r="Y30" s="4" t="n">
-        <v>23.58</v>
+        <v>12.85</v>
       </c>
       <c r="Z30" s="4" t="n">
-        <v>26.53</v>
+        <v>14</v>
       </c>
       <c r="AA30" s="14" t="n">
-        <v>-11.12</v>
+        <v>-8.210000000000001</v>
       </c>
       <c r="AB30" s="4" t="n">
-        <v>23.52</v>
+        <v>12.7</v>
       </c>
       <c r="AC30" s="4" t="n">
-        <v>27.69</v>
+        <v>14.55</v>
       </c>
       <c r="AD30" s="4" t="n">
-        <v>23.52</v>
+        <v>12.7</v>
       </c>
       <c r="AE30" s="4" t="n">
-        <v>25.95</v>
+        <v>13.62</v>
       </c>
       <c r="AF30" s="2" t="inlineStr">
         <is>
@@ -13400,21 +13456,21 @@
       </c>
       <c r="AH30" s="2" t="inlineStr">
         <is>
-          <t>中阴线</t>
+          <t>小阴线</t>
         </is>
       </c>
       <c r="AI30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>2.6</v>
+        <v>1.55</v>
       </c>
       <c r="AK30" s="4" t="n">
-        <v>33.76</v>
-      </c>
-      <c r="AL30" s="20" t="inlineStr">
-        <is>
-          <t>强趋势</t>
+        <v>23.76</v>
+      </c>
+      <c r="AL30" s="19" t="inlineStr">
+        <is>
+          <t>趋势形成中</t>
         </is>
       </c>
       <c r="AM30" s="2" t="inlineStr">
@@ -13423,10 +13479,10 @@
         </is>
       </c>
       <c r="AN30" s="4" t="n">
-        <v>23.52</v>
+        <v>12.7</v>
       </c>
       <c r="AO30" s="4" t="n">
-        <v>0.25</v>
+        <v>1.17</v>
       </c>
       <c r="AP30" s="8" t="inlineStr">
         <is>
@@ -13439,19 +13495,19 @@
         </is>
       </c>
       <c r="AR30" s="4" t="n">
-        <v>0.802</v>
+        <v>0.896</v>
       </c>
       <c r="AS30" s="4" t="n">
-        <v>0.954</v>
+        <v>0.972</v>
       </c>
       <c r="AT30" s="4" t="n">
-        <v>0.909</v>
+        <v>0.946</v>
       </c>
       <c r="AU30" s="4" t="n">
-        <v>0.86</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="AV30" s="4" t="n">
-        <v>0.802</v>
+        <v>0.896</v>
       </c>
       <c r="AW30" s="8" t="inlineStr">
         <is>
@@ -13462,14 +13518,14 @@
         <v>-5</v>
       </c>
       <c r="AY30" s="4" t="n">
-        <v>2.4</v>
+        <v>1.82</v>
       </c>
       <c r="AZ30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="BA30" s="2" t="inlineStr">
         <is>
-          <t>主板</t>
+          <t>科创/创业板</t>
         </is>
       </c>
       <c r="BB30" s="2" t="inlineStr">
@@ -13478,7 +13534,7 @@
         </is>
       </c>
       <c r="BC30" s="4" t="n">
-        <v>25.83</v>
+        <v>23</v>
       </c>
       <c r="BD30" s="8" t="inlineStr">
         <is>
@@ -13486,24 +13542,24 @@
         </is>
       </c>
       <c r="BE30" s="4" t="n">
-        <v>18.21</v>
+        <v>11.03</v>
       </c>
       <c r="BF30" s="4" t="n">
-        <v>22.34</v>
+        <v>15.89</v>
       </c>
       <c r="BG30" s="4" t="n">
-        <v>9.960000000000001</v>
+        <v>1.31</v>
       </c>
       <c r="BH30" s="8" t="inlineStr">
         <is>
-          <t>偏空(低位)</t>
+          <t>低位钝化</t>
         </is>
       </c>
       <c r="BI30" s="4" t="n">
-        <v>-30.42</v>
+        <v>-20.92</v>
       </c>
       <c r="BJ30" s="4" t="n">
-        <v>37.92</v>
+        <v>17.42</v>
       </c>
       <c r="BK30" s="2" t="inlineStr">
         <is>
@@ -13523,33 +13579,33 @@
         </is>
       </c>
       <c r="BP30" s="4" t="n">
-        <v>24.826</v>
+        <v>13.12</v>
       </c>
       <c r="BQ30" s="4" t="n">
-        <v>24.894</v>
+        <v>13.273</v>
       </c>
       <c r="BR30" s="4" t="n">
-        <v>25.579</v>
+        <v>13.559</v>
       </c>
       <c r="BS30" s="4" t="n">
-        <v>26.685</v>
+        <v>13.924</v>
       </c>
       <c r="BT30" s="4" t="n">
-        <v>29.449</v>
+        <v>14.579</v>
       </c>
       <c r="BU30" s="4" t="n">
         <v>0</v>
       </c>
       <c r="BV30" s="4" t="n">
-        <v>-5.02</v>
-      </c>
-      <c r="BW30" s="8" t="inlineStr">
-        <is>
-          <t>极度超卖</t>
+        <v>-2.06</v>
+      </c>
+      <c r="BW30" s="20" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="BX30" s="4" t="n">
-        <v>-7.82</v>
+        <v>-5.23</v>
       </c>
       <c r="BY30" s="8" t="inlineStr">
         <is>
@@ -13557,29 +13613,29 @@
         </is>
       </c>
       <c r="BZ30" s="4" t="n">
-        <v>-11.63</v>
-      </c>
-      <c r="CA30" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
+        <v>-7.71</v>
+      </c>
+      <c r="CA30" s="20" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="CB30" s="4" t="n">
-        <v>-19.93</v>
-      </c>
-      <c r="CC30" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
+        <v>-11.86</v>
+      </c>
+      <c r="CC30" s="20" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="CD30" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CE30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="CF30" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="CG30" s="2" t="n">
         <v>5</v>
@@ -13610,10 +13666,10 @@
         </is>
       </c>
       <c r="CO30" s="4" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="CP30" s="4" t="n">
-        <v>13.5</v>
+        <v>31.6</v>
       </c>
       <c r="CQ30" s="2" t="inlineStr">
         <is>
@@ -13624,16 +13680,16 @@
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>SZ000919</t>
+          <t>SZ002240</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>金陵药业</t>
+          <t>盛新锂能</t>
         </is>
       </c>
       <c r="C31" s="11" t="n">
-        <v>6.53</v>
+        <v>23.58</v>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
@@ -13641,31 +13697,31 @@
         </is>
       </c>
       <c r="E31" s="11" t="n">
-        <v>6.67</v>
+        <v>25.35</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>6.65</v>
+        <v>24.5</v>
       </c>
       <c r="G31" s="11" t="n">
-        <v>6.7</v>
+        <v>25.09</v>
       </c>
       <c r="H31" s="11" t="n">
-        <v>6.52</v>
+        <v>23.52</v>
       </c>
       <c r="I31" s="11" t="n">
-        <v>6.58</v>
+        <v>24.06</v>
       </c>
       <c r="J31" s="16" t="n">
-        <v>-2.1</v>
+        <v>-6.98</v>
       </c>
       <c r="K31" s="11" t="n">
-        <v>2.7</v>
+        <v>6.19</v>
       </c>
       <c r="L31" s="11" t="n">
-        <v>1.06</v>
+        <v>1.35</v>
       </c>
       <c r="M31" s="11" t="n">
-        <v>0.64</v>
+        <v>7.9</v>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
@@ -13673,10 +13729,10 @@
         </is>
       </c>
       <c r="O31" s="11" t="n">
-        <v>1.56</v>
+        <v>3.58</v>
       </c>
       <c r="P31" s="11" t="n">
-        <v>9.68</v>
+        <v>32.65</v>
       </c>
       <c r="Q31" s="11" t="n">
         <v>0</v>
@@ -13690,42 +13746,42 @@
       <c r="T31" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="U31" s="12" t="n">
-        <v>0.46</v>
+      <c r="U31" s="16" t="n">
+        <v>-6.21</v>
       </c>
       <c r="V31" s="11" t="n">
-        <v>2.9</v>
+        <v>5.53</v>
       </c>
       <c r="W31" s="11" t="n">
-        <v>6.57</v>
+        <v>24.69</v>
       </c>
       <c r="X31" s="11" t="n">
-        <v>6.65</v>
+        <v>24.5</v>
       </c>
       <c r="Y31" s="11" t="n">
-        <v>6.53</v>
+        <v>23.58</v>
       </c>
       <c r="Z31" s="11" t="n">
-        <v>6.56</v>
+        <v>26.53</v>
       </c>
       <c r="AA31" s="16" t="n">
-        <v>-0.46</v>
+        <v>-11.12</v>
       </c>
       <c r="AB31" s="11" t="n">
-        <v>6.36</v>
+        <v>23.52</v>
       </c>
       <c r="AC31" s="11" t="n">
-        <v>6.74</v>
+        <v>27.69</v>
       </c>
       <c r="AD31" s="11" t="n">
-        <v>6.36</v>
+        <v>23.52</v>
       </c>
       <c r="AE31" s="11" t="n">
-        <v>6.7</v>
+        <v>25.95</v>
       </c>
       <c r="AF31" s="9" t="inlineStr">
         <is>
-          <t>是（最近金叉）</t>
+          <t>否</t>
         </is>
       </c>
       <c r="AG31" s="9" t="inlineStr">
@@ -13742,14 +13798,14 @@
         <v>0</v>
       </c>
       <c r="AJ31" s="11" t="n">
-        <v>4.86</v>
+        <v>2.6</v>
       </c>
       <c r="AK31" s="11" t="n">
-        <v>14.62</v>
-      </c>
-      <c r="AL31" s="8" t="inlineStr">
-        <is>
-          <t>无趋势</t>
+        <v>33.76</v>
+      </c>
+      <c r="AL31" s="20" t="inlineStr">
+        <is>
+          <t>强趋势</t>
         </is>
       </c>
       <c r="AM31" s="9" t="inlineStr">
@@ -13758,10 +13814,10 @@
         </is>
       </c>
       <c r="AN31" s="11" t="n">
-        <v>6.36</v>
+        <v>23.52</v>
       </c>
       <c r="AO31" s="11" t="n">
-        <v>2.6</v>
+        <v>0.25</v>
       </c>
       <c r="AP31" s="8" t="inlineStr">
         <is>
@@ -13774,30 +13830,30 @@
         </is>
       </c>
       <c r="AR31" s="11" t="n">
-        <v>1.157</v>
+        <v>0.802</v>
       </c>
       <c r="AS31" s="11" t="n">
-        <v>1.029</v>
+        <v>0.954</v>
       </c>
       <c r="AT31" s="11" t="n">
-        <v>1.027</v>
+        <v>0.909</v>
       </c>
       <c r="AU31" s="11" t="n">
-        <v>1.056</v>
+        <v>0.86</v>
       </c>
       <c r="AV31" s="11" t="n">
-        <v>1.157</v>
-      </c>
-      <c r="AW31" s="20" t="inlineStr">
-        <is>
-          <t>总体偏强</t>
+        <v>0.802</v>
+      </c>
+      <c r="AW31" s="8" t="inlineStr">
+        <is>
+          <t>总体偏弱</t>
         </is>
       </c>
       <c r="AX31" s="9" t="n">
-        <v>10</v>
+        <v>-5</v>
       </c>
       <c r="AY31" s="11" t="n">
-        <v>1.51</v>
+        <v>2.4</v>
       </c>
       <c r="AZ31" s="9" t="n">
         <v>0</v>
@@ -13813,32 +13869,32 @@
         </is>
       </c>
       <c r="BC31" s="11" t="n">
-        <v>47.37</v>
-      </c>
-      <c r="BD31" s="19" t="inlineStr">
-        <is>
-          <t>偏弱区</t>
+        <v>25.83</v>
+      </c>
+      <c r="BD31" s="8" t="inlineStr">
+        <is>
+          <t>超卖区</t>
         </is>
       </c>
       <c r="BE31" s="11" t="n">
-        <v>48.98</v>
+        <v>18.21</v>
       </c>
       <c r="BF31" s="11" t="n">
-        <v>43.13</v>
+        <v>22.34</v>
       </c>
       <c r="BG31" s="11" t="n">
-        <v>60.68</v>
-      </c>
-      <c r="BH31" s="20" t="inlineStr">
-        <is>
-          <t>偏多</t>
+        <v>9.960000000000001</v>
+      </c>
+      <c r="BH31" s="8" t="inlineStr">
+        <is>
+          <t>偏空(低位)</t>
         </is>
       </c>
       <c r="BI31" s="11" t="n">
-        <v>-9.359999999999999</v>
+        <v>-30.42</v>
       </c>
       <c r="BJ31" s="11" t="n">
-        <v>30.18</v>
+        <v>37.92</v>
       </c>
       <c r="BK31" s="9" t="inlineStr">
         <is>
@@ -13850,65 +13906,61 @@
           <t>否</t>
         </is>
       </c>
-      <c r="BM31" s="9" t="inlineStr">
-        <is>
-          <t>MACD金叉</t>
-        </is>
-      </c>
+      <c r="BM31" s="9" t="inlineStr"/>
       <c r="BN31" s="9" t="inlineStr"/>
       <c r="BO31" s="7" t="inlineStr">
         <is>
-          <t>弱市</t>
+          <t>深回撤|弱市</t>
         </is>
       </c>
       <c r="BP31" s="11" t="n">
-        <v>6.526</v>
+        <v>24.826</v>
       </c>
       <c r="BQ31" s="11" t="n">
-        <v>6.501</v>
+        <v>24.894</v>
       </c>
       <c r="BR31" s="11" t="n">
-        <v>6.537</v>
+        <v>25.579</v>
       </c>
       <c r="BS31" s="11" t="n">
-        <v>6.545</v>
+        <v>26.685</v>
       </c>
       <c r="BT31" s="11" t="n">
-        <v>6.511</v>
+        <v>29.449</v>
       </c>
       <c r="BU31" s="11" t="n">
         <v>0</v>
       </c>
       <c r="BV31" s="11" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="BW31" s="20" t="inlineStr">
-        <is>
-          <t>中性区间</t>
+        <v>-5.02</v>
+      </c>
+      <c r="BW31" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
         </is>
       </c>
       <c r="BX31" s="11" t="n">
-        <v>-0.11</v>
-      </c>
-      <c r="BY31" s="20" t="inlineStr">
-        <is>
-          <t>中性区间</t>
+        <v>-7.82</v>
+      </c>
+      <c r="BY31" s="8" t="inlineStr">
+        <is>
+          <t>超卖偏弱</t>
         </is>
       </c>
       <c r="BZ31" s="11" t="n">
-        <v>-0.23</v>
-      </c>
-      <c r="CA31" s="20" t="inlineStr">
-        <is>
-          <t>中性区间</t>
+        <v>-11.63</v>
+      </c>
+      <c r="CA31" s="8" t="inlineStr">
+        <is>
+          <t>超卖偏弱</t>
         </is>
       </c>
       <c r="CB31" s="11" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="CC31" s="20" t="inlineStr">
-        <is>
-          <t>中性区间</t>
+        <v>-19.93</v>
+      </c>
+      <c r="CC31" s="8" t="inlineStr">
+        <is>
+          <t>超卖偏弱</t>
         </is>
       </c>
       <c r="CD31" s="9" t="n">
@@ -13918,7 +13970,7 @@
         <v>0</v>
       </c>
       <c r="CF31" s="9" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="CG31" s="9" t="n">
         <v>5</v>
@@ -13930,7 +13982,7 @@
         <v>0</v>
       </c>
       <c r="CJ31" s="9" t="n">
-        <v>10</v>
+        <v>-5</v>
       </c>
       <c r="CK31" s="9" t="n">
         <v>0</v>
@@ -13949,10 +14001,10 @@
         </is>
       </c>
       <c r="CO31" s="11" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="CP31" s="11" t="n">
-        <v>73</v>
+        <v>13.2</v>
       </c>
       <c r="CQ31" s="9" t="inlineStr">
         <is>
@@ -13963,16 +14015,16 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>SZ002402</t>
+          <t>SZ000919</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>和而泰</t>
+          <t>金陵药业</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>17.21</v>
+        <v>6.53</v>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
@@ -13980,31 +14032,31 @@
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>17.54</v>
+        <v>6.67</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>17.49</v>
+        <v>6.65</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>17.64</v>
+        <v>6.7</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>17.17</v>
+        <v>6.52</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>17.34</v>
+        <v>6.58</v>
       </c>
       <c r="J32" s="14" t="n">
-        <v>-1.88</v>
+        <v>-2.1</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>2.68</v>
+        <v>2.7</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>0.83</v>
+        <v>1.06</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>2.37</v>
+        <v>0.64</v>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
@@ -14012,10 +14064,10 @@
         </is>
       </c>
       <c r="O32" s="4" t="n">
-        <v>1.67</v>
+        <v>1.56</v>
       </c>
       <c r="P32" s="4" t="n">
-        <v>13.66</v>
+        <v>9.68</v>
       </c>
       <c r="Q32" s="4" t="n">
         <v>0</v>
@@ -14029,42 +14081,42 @@
       <c r="T32" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="U32" s="14" t="n">
-        <v>-1.77</v>
+      <c r="U32" s="5" t="n">
+        <v>0.46</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>3.45</v>
+        <v>2.9</v>
       </c>
       <c r="W32" s="4" t="n">
-        <v>17.42</v>
+        <v>6.57</v>
       </c>
       <c r="X32" s="4" t="n">
-        <v>17.49</v>
+        <v>6.65</v>
       </c>
       <c r="Y32" s="4" t="n">
-        <v>17.21</v>
+        <v>6.53</v>
       </c>
       <c r="Z32" s="4" t="n">
-        <v>18.29</v>
+        <v>6.56</v>
       </c>
       <c r="AA32" s="14" t="n">
-        <v>-5.9</v>
+        <v>-0.46</v>
       </c>
       <c r="AB32" s="4" t="n">
-        <v>16.95</v>
+        <v>6.36</v>
       </c>
       <c r="AC32" s="4" t="n">
-        <v>19.24</v>
+        <v>6.74</v>
       </c>
       <c r="AD32" s="4" t="n">
-        <v>16.95</v>
+        <v>6.36</v>
       </c>
       <c r="AE32" s="4" t="n">
-        <v>18.05</v>
+        <v>6.7</v>
       </c>
       <c r="AF32" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是（最近金叉）</t>
         </is>
       </c>
       <c r="AG32" s="2" t="inlineStr">
@@ -14081,14 +14133,14 @@
         <v>0</v>
       </c>
       <c r="AJ32" s="4" t="n">
-        <v>3.53</v>
+        <v>4.86</v>
       </c>
       <c r="AK32" s="4" t="n">
-        <v>35.1</v>
-      </c>
-      <c r="AL32" s="20" t="inlineStr">
-        <is>
-          <t>强趋势</t>
+        <v>14.62</v>
+      </c>
+      <c r="AL32" s="8" t="inlineStr">
+        <is>
+          <t>无趋势</t>
         </is>
       </c>
       <c r="AM32" s="2" t="inlineStr">
@@ -14097,47 +14149,47 @@
         </is>
       </c>
       <c r="AN32" s="4" t="n">
-        <v>16.95</v>
+        <v>6.36</v>
       </c>
       <c r="AO32" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AP32" s="8" t="inlineStr">
+        <is>
+          <t>极低波动盘整</t>
+        </is>
+      </c>
+      <c r="AQ32" s="2" t="inlineStr">
+        <is>
+          <t>下降</t>
+        </is>
+      </c>
+      <c r="AR32" s="4" t="n">
+        <v>1.157</v>
+      </c>
+      <c r="AS32" s="4" t="n">
+        <v>1.029</v>
+      </c>
+      <c r="AT32" s="4" t="n">
+        <v>1.027</v>
+      </c>
+      <c r="AU32" s="4" t="n">
+        <v>1.056</v>
+      </c>
+      <c r="AV32" s="4" t="n">
+        <v>1.157</v>
+      </c>
+      <c r="AW32" s="20" t="inlineStr">
+        <is>
+          <t>总体偏强</t>
+        </is>
+      </c>
+      <c r="AX32" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AY32" s="4" t="n">
         <v>1.51</v>
       </c>
-      <c r="AP32" s="8" t="inlineStr">
-        <is>
-          <t>极低波动盘整</t>
-        </is>
-      </c>
-      <c r="AQ32" s="2" t="inlineStr">
-        <is>
-          <t>下降</t>
-        </is>
-      </c>
-      <c r="AR32" s="4" t="n">
-        <v>0.757</v>
-      </c>
-      <c r="AS32" s="4" t="n">
-        <v>0.979</v>
-      </c>
-      <c r="AT32" s="4" t="n">
-        <v>0.956</v>
-      </c>
-      <c r="AU32" s="4" t="n">
-        <v>0.974</v>
-      </c>
-      <c r="AV32" s="4" t="n">
-        <v>0.757</v>
-      </c>
-      <c r="AW32" s="8" t="inlineStr">
-        <is>
-          <t>总体偏弱</t>
-        </is>
-      </c>
-      <c r="AX32" s="2" t="n">
-        <v>-5</v>
-      </c>
-      <c r="AY32" s="4" t="n">
-        <v>1.95</v>
-      </c>
       <c r="AZ32" s="2" t="n">
         <v>0</v>
       </c>
@@ -14152,7 +14204,7 @@
         </is>
       </c>
       <c r="BC32" s="4" t="n">
-        <v>32.04</v>
+        <v>47.37</v>
       </c>
       <c r="BD32" s="19" t="inlineStr">
         <is>
@@ -14160,24 +14212,24 @@
         </is>
       </c>
       <c r="BE32" s="4" t="n">
-        <v>17.6</v>
+        <v>48.98</v>
       </c>
       <c r="BF32" s="4" t="n">
-        <v>25.38</v>
+        <v>43.13</v>
       </c>
       <c r="BG32" s="4" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="BH32" s="8" t="inlineStr">
-        <is>
-          <t>偏空(低位)</t>
+        <v>60.68</v>
+      </c>
+      <c r="BH32" s="20" t="inlineStr">
+        <is>
+          <t>偏多</t>
         </is>
       </c>
       <c r="BI32" s="4" t="n">
-        <v>-30.91</v>
+        <v>-9.359999999999999</v>
       </c>
       <c r="BJ32" s="4" t="n">
-        <v>22.29</v>
+        <v>30.18</v>
       </c>
       <c r="BK32" s="2" t="inlineStr">
         <is>
@@ -14189,33 +14241,37 @@
           <t>否</t>
         </is>
       </c>
-      <c r="BM32" s="2" t="inlineStr"/>
+      <c r="BM32" s="2" t="inlineStr">
+        <is>
+          <t>MACD金叉</t>
+        </is>
+      </c>
       <c r="BN32" s="2" t="inlineStr"/>
       <c r="BO32" s="7" t="inlineStr">
         <is>
-          <t>深回撤|弱市</t>
+          <t>弱市</t>
         </is>
       </c>
       <c r="BP32" s="4" t="n">
-        <v>17.54</v>
+        <v>6.526</v>
       </c>
       <c r="BQ32" s="4" t="n">
-        <v>17.697</v>
+        <v>6.501</v>
       </c>
       <c r="BR32" s="4" t="n">
-        <v>18.061</v>
+        <v>6.537</v>
       </c>
       <c r="BS32" s="4" t="n">
-        <v>18.28</v>
+        <v>6.545</v>
       </c>
       <c r="BT32" s="4" t="n">
-        <v>19.744</v>
+        <v>6.511</v>
       </c>
       <c r="BU32" s="4" t="n">
         <v>0</v>
       </c>
       <c r="BV32" s="4" t="n">
-        <v>-1.88</v>
+        <v>0.06</v>
       </c>
       <c r="BW32" s="20" t="inlineStr">
         <is>
@@ -14223,7 +14279,7 @@
         </is>
       </c>
       <c r="BX32" s="4" t="n">
-        <v>-4.71</v>
+        <v>-0.11</v>
       </c>
       <c r="BY32" s="20" t="inlineStr">
         <is>
@@ -14231,7 +14287,7 @@
         </is>
       </c>
       <c r="BZ32" s="4" t="n">
-        <v>-5.85</v>
+        <v>-0.23</v>
       </c>
       <c r="CA32" s="20" t="inlineStr">
         <is>
@@ -14239,7 +14295,7 @@
         </is>
       </c>
       <c r="CB32" s="4" t="n">
-        <v>-12.83</v>
+        <v>0.29</v>
       </c>
       <c r="CC32" s="20" t="inlineStr">
         <is>
@@ -14253,7 +14309,7 @@
         <v>0</v>
       </c>
       <c r="CF32" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="CG32" s="2" t="n">
         <v>5</v>
@@ -14265,7 +14321,7 @@
         <v>0</v>
       </c>
       <c r="CJ32" s="2" t="n">
-        <v>-5</v>
+        <v>10</v>
       </c>
       <c r="CK32" s="2" t="n">
         <v>0</v>
@@ -14284,10 +14340,10 @@
         </is>
       </c>
       <c r="CO32" s="4" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="CP32" s="4" t="n">
-        <v>2.7</v>
+        <v>73.7</v>
       </c>
       <c r="CQ32" s="2" t="inlineStr">
         <is>
@@ -14298,16 +14354,16 @@
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>SZ002475</t>
+          <t>SZ002402</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>立讯精密</t>
+          <t>和而泰</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>46.32</v>
+        <v>17.21</v>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
@@ -14315,31 +14371,31 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>47.59</v>
+        <v>17.54</v>
       </c>
       <c r="F33" s="11" t="n">
-        <v>46.6</v>
+        <v>17.49</v>
       </c>
       <c r="G33" s="11" t="n">
-        <v>48.1</v>
+        <v>17.64</v>
       </c>
       <c r="H33" s="11" t="n">
-        <v>46.19</v>
+        <v>17.17</v>
       </c>
       <c r="I33" s="11" t="n">
-        <v>46.87</v>
+        <v>17.34</v>
       </c>
       <c r="J33" s="16" t="n">
-        <v>-2.67</v>
+        <v>-1.88</v>
       </c>
       <c r="K33" s="11" t="n">
-        <v>4.01</v>
+        <v>2.68</v>
       </c>
       <c r="L33" s="11" t="n">
-        <v>1.48</v>
+        <v>0.83</v>
       </c>
       <c r="M33" s="11" t="n">
-        <v>50.99</v>
+        <v>2.37</v>
       </c>
       <c r="N33" s="9" t="inlineStr">
         <is>
@@ -14347,10 +14403,10 @@
         </is>
       </c>
       <c r="O33" s="11" t="n">
-        <v>1.48</v>
+        <v>1.67</v>
       </c>
       <c r="P33" s="11" t="n">
-        <v>108.76</v>
+        <v>13.66</v>
       </c>
       <c r="Q33" s="11" t="n">
         <v>0</v>
@@ -14365,37 +14421,37 @@
         <v>0</v>
       </c>
       <c r="U33" s="16" t="n">
-        <v>-4.36</v>
+        <v>-1.77</v>
       </c>
       <c r="V33" s="11" t="n">
-        <v>4.28</v>
+        <v>3.45</v>
       </c>
       <c r="W33" s="11" t="n">
-        <v>47.45</v>
+        <v>17.42</v>
       </c>
       <c r="X33" s="11" t="n">
-        <v>46.6</v>
+        <v>17.49</v>
       </c>
       <c r="Y33" s="11" t="n">
-        <v>46.32</v>
+        <v>17.21</v>
       </c>
       <c r="Z33" s="11" t="n">
-        <v>52.36</v>
+        <v>18.29</v>
       </c>
       <c r="AA33" s="16" t="n">
-        <v>-11.54</v>
+        <v>-5.9</v>
       </c>
       <c r="AB33" s="11" t="n">
-        <v>46.02</v>
+        <v>16.95</v>
       </c>
       <c r="AC33" s="11" t="n">
-        <v>55.8</v>
+        <v>19.24</v>
       </c>
       <c r="AD33" s="11" t="n">
-        <v>46.02</v>
+        <v>16.95</v>
       </c>
       <c r="AE33" s="11" t="n">
-        <v>50.88</v>
+        <v>18.05</v>
       </c>
       <c r="AF33" s="9" t="inlineStr">
         <is>
@@ -14409,17 +14465,17 @@
       </c>
       <c r="AH33" s="9" t="inlineStr">
         <is>
-          <t>流星线 (看跌)</t>
+          <t>中阴线</t>
         </is>
       </c>
       <c r="AI33" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AJ33" s="11" t="n">
-        <v>2.22</v>
+        <v>3.53</v>
       </c>
       <c r="AK33" s="11" t="n">
-        <v>34.5</v>
+        <v>35.1</v>
       </c>
       <c r="AL33" s="20" t="inlineStr">
         <is>
@@ -14432,10 +14488,10 @@
         </is>
       </c>
       <c r="AN33" s="11" t="n">
-        <v>46.02</v>
+        <v>16.95</v>
       </c>
       <c r="AO33" s="11" t="n">
-        <v>0.65</v>
+        <v>1.51</v>
       </c>
       <c r="AP33" s="8" t="inlineStr">
         <is>
@@ -14448,19 +14504,19 @@
         </is>
       </c>
       <c r="AR33" s="11" t="n">
-        <v>0.862</v>
+        <v>0.757</v>
       </c>
       <c r="AS33" s="11" t="n">
-        <v>0.931</v>
+        <v>0.979</v>
       </c>
       <c r="AT33" s="11" t="n">
-        <v>0.901</v>
+        <v>0.956</v>
       </c>
       <c r="AU33" s="11" t="n">
-        <v>0.884</v>
+        <v>0.974</v>
       </c>
       <c r="AV33" s="11" t="n">
-        <v>0.862</v>
+        <v>0.757</v>
       </c>
       <c r="AW33" s="8" t="inlineStr">
         <is>
@@ -14471,7 +14527,7 @@
         <v>-5</v>
       </c>
       <c r="AY33" s="11" t="n">
-        <v>1.11</v>
+        <v>1.95</v>
       </c>
       <c r="AZ33" s="9" t="n">
         <v>0</v>
@@ -14487,32 +14543,32 @@
         </is>
       </c>
       <c r="BC33" s="11" t="n">
-        <v>28.97</v>
-      </c>
-      <c r="BD33" s="8" t="inlineStr">
-        <is>
-          <t>超卖区</t>
+        <v>32.04</v>
+      </c>
+      <c r="BD33" s="19" t="inlineStr">
+        <is>
+          <t>偏弱区</t>
         </is>
       </c>
       <c r="BE33" s="11" t="n">
-        <v>11.78</v>
+        <v>17.6</v>
       </c>
       <c r="BF33" s="11" t="n">
-        <v>19.47</v>
+        <v>25.38</v>
       </c>
       <c r="BG33" s="11" t="n">
-        <v>-3.59</v>
+        <v>2.05</v>
       </c>
       <c r="BH33" s="8" t="inlineStr">
         <is>
-          <t>极度超卖</t>
+          <t>偏空(低位)</t>
         </is>
       </c>
       <c r="BI33" s="11" t="n">
-        <v>-26.35</v>
+        <v>-30.91</v>
       </c>
       <c r="BJ33" s="11" t="n">
-        <v>38.44</v>
+        <v>22.29</v>
       </c>
       <c r="BK33" s="9" t="inlineStr">
         <is>
@@ -14532,53 +14588,53 @@
         </is>
       </c>
       <c r="BP33" s="11" t="n">
-        <v>48.434</v>
+        <v>17.54</v>
       </c>
       <c r="BQ33" s="11" t="n">
-        <v>49.156</v>
+        <v>17.697</v>
       </c>
       <c r="BR33" s="11" t="n">
-        <v>50.774</v>
+        <v>18.061</v>
       </c>
       <c r="BS33" s="11" t="n">
-        <v>52.398</v>
+        <v>18.28</v>
       </c>
       <c r="BT33" s="11" t="n">
-        <v>55.772</v>
+        <v>19.744</v>
       </c>
       <c r="BU33" s="11" t="n">
         <v>0</v>
       </c>
       <c r="BV33" s="11" t="n">
-        <v>-4.36</v>
-      </c>
-      <c r="BW33" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
+        <v>-1.88</v>
+      </c>
+      <c r="BW33" s="20" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="BX33" s="11" t="n">
-        <v>-8.77</v>
-      </c>
-      <c r="BY33" s="8" t="inlineStr">
-        <is>
-          <t>极度超卖</t>
+        <v>-4.71</v>
+      </c>
+      <c r="BY33" s="20" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="BZ33" s="11" t="n">
-        <v>-11.6</v>
-      </c>
-      <c r="CA33" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
+        <v>-5.85</v>
+      </c>
+      <c r="CA33" s="20" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="CB33" s="11" t="n">
-        <v>-16.95</v>
-      </c>
-      <c r="CC33" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
+        <v>-12.83</v>
+      </c>
+      <c r="CC33" s="20" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="CD33" s="9" t="n">
@@ -14619,10 +14675,10 @@
         </is>
       </c>
       <c r="CO33" s="11" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="CP33" s="11" t="n">
-        <v>27</v>
+        <v>2.6</v>
       </c>
       <c r="CQ33" s="9" t="inlineStr">
         <is>
@@ -14633,16 +14689,16 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SZ002241</t>
+          <t>SZ002475</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>歌尔股份</t>
+          <t>立讯精密</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>20.85</v>
+        <v>46.32</v>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
@@ -14650,31 +14706,31 @@
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>21.51</v>
+        <v>47.59</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>21.3</v>
+        <v>46.6</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>21.4</v>
+        <v>48.1</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>20.81</v>
+        <v>46.19</v>
       </c>
       <c r="I34" s="4" t="n">
-        <v>21.02</v>
+        <v>46.87</v>
       </c>
       <c r="J34" s="14" t="n">
-        <v>-3.07</v>
+        <v>-2.67</v>
       </c>
       <c r="K34" s="4" t="n">
-        <v>2.74</v>
+        <v>4.01</v>
       </c>
       <c r="L34" s="4" t="n">
-        <v>0.89</v>
+        <v>1.48</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>12.72</v>
+        <v>50.99</v>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
@@ -14682,10 +14738,10 @@
         </is>
       </c>
       <c r="O34" s="4" t="n">
-        <v>1.92</v>
+        <v>1.48</v>
       </c>
       <c r="P34" s="4" t="n">
-        <v>60.42</v>
+        <v>108.76</v>
       </c>
       <c r="Q34" s="4" t="n">
         <v>0</v>
@@ -14700,37 +14756,37 @@
         <v>0</v>
       </c>
       <c r="U34" s="14" t="n">
-        <v>-3.92</v>
+        <v>-4.36</v>
       </c>
       <c r="V34" s="4" t="n">
-        <v>4.32</v>
+        <v>4.28</v>
       </c>
       <c r="W34" s="4" t="n">
-        <v>21.35</v>
+        <v>47.45</v>
       </c>
       <c r="X34" s="4" t="n">
-        <v>21.3</v>
+        <v>46.6</v>
       </c>
       <c r="Y34" s="4" t="n">
-        <v>20.85</v>
+        <v>46.32</v>
       </c>
       <c r="Z34" s="4" t="n">
-        <v>23.13</v>
+        <v>52.36</v>
       </c>
       <c r="AA34" s="14" t="n">
-        <v>-9.859999999999999</v>
+        <v>-11.54</v>
       </c>
       <c r="AB34" s="4" t="n">
-        <v>20.81</v>
+        <v>46.02</v>
       </c>
       <c r="AC34" s="4" t="n">
-        <v>25.48</v>
+        <v>55.8</v>
       </c>
       <c r="AD34" s="4" t="n">
-        <v>20.81</v>
+        <v>46.02</v>
       </c>
       <c r="AE34" s="4" t="n">
-        <v>23.43</v>
+        <v>50.88</v>
       </c>
       <c r="AF34" s="2" t="inlineStr">
         <is>
@@ -14744,21 +14800,21 @@
       </c>
       <c r="AH34" s="2" t="inlineStr">
         <is>
-          <t>小阴线</t>
+          <t>流星线 (看跌)</t>
         </is>
       </c>
       <c r="AI34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>2.53</v>
+        <v>2.22</v>
       </c>
       <c r="AK34" s="4" t="n">
-        <v>16.95</v>
-      </c>
-      <c r="AL34" s="8" t="inlineStr">
-        <is>
-          <t>无趋势</t>
+        <v>34.5</v>
+      </c>
+      <c r="AL34" s="20" t="inlineStr">
+        <is>
+          <t>强趋势</t>
         </is>
       </c>
       <c r="AM34" s="2" t="inlineStr">
@@ -14767,10 +14823,10 @@
         </is>
       </c>
       <c r="AN34" s="4" t="n">
-        <v>20.81</v>
+        <v>46.02</v>
       </c>
       <c r="AO34" s="4" t="n">
-        <v>0.19</v>
+        <v>0.65</v>
       </c>
       <c r="AP34" s="8" t="inlineStr">
         <is>
@@ -14783,30 +14839,30 @@
         </is>
       </c>
       <c r="AR34" s="4" t="n">
-        <v>1.046</v>
+        <v>0.862</v>
       </c>
       <c r="AS34" s="4" t="n">
-        <v>0.919</v>
+        <v>0.931</v>
       </c>
       <c r="AT34" s="4" t="n">
-        <v>0.927</v>
+        <v>0.901</v>
       </c>
       <c r="AU34" s="4" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.884</v>
       </c>
       <c r="AV34" s="4" t="n">
-        <v>1.046</v>
-      </c>
-      <c r="AW34" s="19" t="inlineStr">
-        <is>
-          <t>强弱不明，震荡</t>
+        <v>0.862</v>
+      </c>
+      <c r="AW34" s="8" t="inlineStr">
+        <is>
+          <t>总体偏弱</t>
         </is>
       </c>
       <c r="AX34" s="2" t="n">
-        <v>5</v>
+        <v>-5</v>
       </c>
       <c r="AY34" s="4" t="n">
-        <v>2.49</v>
+        <v>1.11</v>
       </c>
       <c r="AZ34" s="2" t="n">
         <v>0</v>
@@ -14822,32 +14878,32 @@
         </is>
       </c>
       <c r="BC34" s="4" t="n">
-        <v>42.19</v>
-      </c>
-      <c r="BD34" s="19" t="inlineStr">
-        <is>
-          <t>偏弱区</t>
+        <v>28.97</v>
+      </c>
+      <c r="BD34" s="8" t="inlineStr">
+        <is>
+          <t>超卖区</t>
         </is>
       </c>
       <c r="BE34" s="4" t="n">
-        <v>17.81</v>
+        <v>11.78</v>
       </c>
       <c r="BF34" s="4" t="n">
-        <v>32.83</v>
+        <v>19.47</v>
       </c>
       <c r="BG34" s="4" t="n">
-        <v>-12.24</v>
-      </c>
-      <c r="BH34" s="19" t="inlineStr">
-        <is>
-          <t>偏空</t>
+        <v>-3.59</v>
+      </c>
+      <c r="BH34" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
         </is>
       </c>
       <c r="BI34" s="4" t="n">
-        <v>-15.38</v>
+        <v>-26.35</v>
       </c>
       <c r="BJ34" s="4" t="n">
-        <v>39.23</v>
+        <v>38.44</v>
       </c>
       <c r="BK34" s="2" t="inlineStr">
         <is>
@@ -14863,45 +14919,45 @@
       <c r="BN34" s="2" t="inlineStr"/>
       <c r="BO34" s="7" t="inlineStr">
         <is>
-          <t>弱市</t>
+          <t>深回撤|弱市</t>
         </is>
       </c>
       <c r="BP34" s="4" t="n">
-        <v>21.97</v>
+        <v>48.434</v>
       </c>
       <c r="BQ34" s="4" t="n">
-        <v>22.42</v>
+        <v>49.156</v>
       </c>
       <c r="BR34" s="4" t="n">
-        <v>22.983</v>
+        <v>50.774</v>
       </c>
       <c r="BS34" s="4" t="n">
-        <v>22.773</v>
+        <v>52.398</v>
       </c>
       <c r="BT34" s="4" t="n">
-        <v>22.92</v>
+        <v>55.772</v>
       </c>
       <c r="BU34" s="4" t="n">
         <v>0</v>
       </c>
       <c r="BV34" s="4" t="n">
-        <v>-5.1</v>
+        <v>-4.36</v>
       </c>
       <c r="BW34" s="8" t="inlineStr">
         <is>
+          <t>超卖偏弱</t>
+        </is>
+      </c>
+      <c r="BX34" s="4" t="n">
+        <v>-8.77</v>
+      </c>
+      <c r="BY34" s="8" t="inlineStr">
+        <is>
           <t>极度超卖</t>
         </is>
       </c>
-      <c r="BX34" s="4" t="n">
-        <v>-9.279999999999999</v>
-      </c>
-      <c r="BY34" s="8" t="inlineStr">
-        <is>
-          <t>极度超卖</t>
-        </is>
-      </c>
       <c r="BZ34" s="4" t="n">
-        <v>-8.44</v>
+        <v>-11.6</v>
       </c>
       <c r="CA34" s="8" t="inlineStr">
         <is>
@@ -14909,11 +14965,11 @@
         </is>
       </c>
       <c r="CB34" s="4" t="n">
-        <v>-9.029999999999999</v>
-      </c>
-      <c r="CC34" s="20" t="inlineStr">
-        <is>
-          <t>中性区间</t>
+        <v>-16.95</v>
+      </c>
+      <c r="CC34" s="8" t="inlineStr">
+        <is>
+          <t>超卖偏弱</t>
         </is>
       </c>
       <c r="CD34" s="2" t="n">
@@ -14923,7 +14979,7 @@
         <v>0</v>
       </c>
       <c r="CF34" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="CG34" s="2" t="n">
         <v>5</v>
@@ -14935,7 +14991,7 @@
         <v>0</v>
       </c>
       <c r="CJ34" s="2" t="n">
-        <v>5</v>
+        <v>-5</v>
       </c>
       <c r="CK34" s="2" t="n">
         <v>0</v>
@@ -14954,10 +15010,10 @@
         </is>
       </c>
       <c r="CO34" s="4" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="CP34" s="4" t="n">
-        <v>56.8</v>
+        <v>26.3</v>
       </c>
       <c r="CQ34" s="2" t="inlineStr">
         <is>
@@ -14968,16 +15024,16 @@
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>SZ300442</t>
+          <t>SZ002241</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>润泽科技</t>
+          <t>歌尔股份</t>
         </is>
       </c>
       <c r="C35" s="11" t="n">
-        <v>57.64</v>
+        <v>20.85</v>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
@@ -14985,170 +15041,170 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>58.63</v>
+        <v>21.51</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>58.49</v>
+        <v>21.3</v>
       </c>
       <c r="G35" s="11" t="n">
-        <v>58.8</v>
+        <v>21.4</v>
       </c>
       <c r="H35" s="11" t="n">
-        <v>57.34</v>
+        <v>20.81</v>
       </c>
       <c r="I35" s="11" t="n">
-        <v>57.93</v>
+        <v>21.02</v>
       </c>
       <c r="J35" s="16" t="n">
-        <v>-1.69</v>
+        <v>-3.07</v>
       </c>
       <c r="K35" s="11" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="L35" s="11" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="M35" s="11" t="n">
+        <v>12.72</v>
+      </c>
+      <c r="N35" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="O35" s="11" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="P35" s="11" t="n">
+        <v>60.42</v>
+      </c>
+      <c r="Q35" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" s="16" t="n">
+        <v>-3.92</v>
+      </c>
+      <c r="V35" s="11" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="W35" s="11" t="n">
+        <v>21.35</v>
+      </c>
+      <c r="X35" s="11" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="Y35" s="11" t="n">
+        <v>20.85</v>
+      </c>
+      <c r="Z35" s="11" t="n">
+        <v>23.13</v>
+      </c>
+      <c r="AA35" s="16" t="n">
+        <v>-9.859999999999999</v>
+      </c>
+      <c r="AB35" s="11" t="n">
+        <v>20.81</v>
+      </c>
+      <c r="AC35" s="11" t="n">
+        <v>25.48</v>
+      </c>
+      <c r="AD35" s="11" t="n">
+        <v>20.81</v>
+      </c>
+      <c r="AE35" s="11" t="n">
+        <v>23.43</v>
+      </c>
+      <c r="AF35" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AG35" s="9" t="inlineStr">
+        <is>
+          <t>无明显形态</t>
+        </is>
+      </c>
+      <c r="AH35" s="9" t="inlineStr">
+        <is>
+          <t>小阴线</t>
+        </is>
+      </c>
+      <c r="AI35" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ35" s="11" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="AK35" s="11" t="n">
+        <v>16.95</v>
+      </c>
+      <c r="AL35" s="8" t="inlineStr">
+        <is>
+          <t>无趋势</t>
+        </is>
+      </c>
+      <c r="AM35" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AN35" s="11" t="n">
+        <v>20.81</v>
+      </c>
+      <c r="AO35" s="11" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="AP35" s="8" t="inlineStr">
+        <is>
+          <t>极低波动盘整</t>
+        </is>
+      </c>
+      <c r="AQ35" s="9" t="inlineStr">
+        <is>
+          <t>下降</t>
+        </is>
+      </c>
+      <c r="AR35" s="11" t="n">
+        <v>1.046</v>
+      </c>
+      <c r="AS35" s="11" t="n">
+        <v>0.919</v>
+      </c>
+      <c r="AT35" s="11" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="AU35" s="11" t="n">
+        <v>0.9429999999999999</v>
+      </c>
+      <c r="AV35" s="11" t="n">
+        <v>1.046</v>
+      </c>
+      <c r="AW35" s="19" t="inlineStr">
+        <is>
+          <t>强弱不明，震荡</t>
+        </is>
+      </c>
+      <c r="AX35" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY35" s="11" t="n">
         <v>2.49</v>
       </c>
-      <c r="L35" s="11" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="M35" s="11" t="n">
-        <v>7.82</v>
-      </c>
-      <c r="N35" s="9" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="O35" s="11" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="P35" s="11" t="n">
-        <v>13.49</v>
-      </c>
-      <c r="Q35" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="S35" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="T35" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="U35" s="16" t="n">
-        <v>-7.67</v>
-      </c>
-      <c r="V35" s="11" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="W35" s="11" t="n">
-        <v>59.57</v>
-      </c>
-      <c r="X35" s="11" t="n">
-        <v>58.49</v>
-      </c>
-      <c r="Y35" s="11" t="n">
-        <v>57.64</v>
-      </c>
-      <c r="Z35" s="11" t="n">
-        <v>63.46</v>
-      </c>
-      <c r="AA35" s="16" t="n">
-        <v>-9.17</v>
-      </c>
-      <c r="AB35" s="11" t="n">
-        <v>55.92</v>
-      </c>
-      <c r="AC35" s="11" t="n">
-        <v>68.52</v>
-      </c>
-      <c r="AD35" s="11" t="n">
-        <v>55.92</v>
-      </c>
-      <c r="AE35" s="11" t="n">
-        <v>66.98999999999999</v>
-      </c>
-      <c r="AF35" s="9" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="AG35" s="9" t="inlineStr">
-        <is>
-          <t>无明显形态</t>
-        </is>
-      </c>
-      <c r="AH35" s="9" t="inlineStr">
-        <is>
-          <t>小阴线</t>
-        </is>
-      </c>
-      <c r="AI35" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ35" s="11" t="n">
-        <v>4.26</v>
-      </c>
-      <c r="AK35" s="11" t="n">
-        <v>19.98</v>
-      </c>
-      <c r="AL35" s="8" t="inlineStr">
-        <is>
-          <t>无趋势</t>
-        </is>
-      </c>
-      <c r="AM35" s="9" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="AN35" s="11" t="n">
-        <v>55.92</v>
-      </c>
-      <c r="AO35" s="11" t="n">
-        <v>2.98</v>
-      </c>
-      <c r="AP35" s="8" t="inlineStr">
-        <is>
-          <t>极低波动盘整</t>
-        </is>
-      </c>
-      <c r="AQ35" s="9" t="inlineStr">
-        <is>
-          <t>上升</t>
-        </is>
-      </c>
-      <c r="AR35" s="11" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="AS35" s="11" t="n">
-        <v>0.888</v>
-      </c>
-      <c r="AT35" s="11" t="n">
-        <v>0.976</v>
-      </c>
-      <c r="AU35" s="11" t="n">
-        <v>0.968</v>
-      </c>
-      <c r="AV35" s="11" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="AW35" s="8" t="inlineStr">
-        <is>
-          <t>总体偏弱</t>
-        </is>
-      </c>
-      <c r="AX35" s="9" t="n">
-        <v>-5</v>
-      </c>
-      <c r="AY35" s="11" t="n">
-        <v>1.26</v>
-      </c>
       <c r="AZ35" s="9" t="n">
         <v>0</v>
       </c>
       <c r="BA35" s="9" t="inlineStr">
         <is>
-          <t>科创/创业板</t>
+          <t>主板</t>
         </is>
       </c>
       <c r="BB35" s="9" t="inlineStr">
@@ -15157,7 +15213,7 @@
         </is>
       </c>
       <c r="BC35" s="11" t="n">
-        <v>43.99</v>
+        <v>42.19</v>
       </c>
       <c r="BD35" s="19" t="inlineStr">
         <is>
@@ -15165,13 +15221,13 @@
         </is>
       </c>
       <c r="BE35" s="11" t="n">
-        <v>27.4</v>
+        <v>17.81</v>
       </c>
       <c r="BF35" s="11" t="n">
-        <v>42.62</v>
+        <v>32.83</v>
       </c>
       <c r="BG35" s="11" t="n">
-        <v>-3.03</v>
+        <v>-12.24</v>
       </c>
       <c r="BH35" s="19" t="inlineStr">
         <is>
@@ -15179,10 +15235,10 @@
         </is>
       </c>
       <c r="BI35" s="11" t="n">
-        <v>-25.29</v>
+        <v>-15.38</v>
       </c>
       <c r="BJ35" s="11" t="n">
-        <v>42.39</v>
+        <v>39.23</v>
       </c>
       <c r="BK35" s="9" t="inlineStr">
         <is>
@@ -15198,29 +15254,29 @@
       <c r="BN35" s="9" t="inlineStr"/>
       <c r="BO35" s="7" t="inlineStr">
         <is>
-          <t>深回撤|弱市</t>
+          <t>弱市</t>
         </is>
       </c>
       <c r="BP35" s="11" t="n">
-        <v>61.696</v>
+        <v>21.97</v>
       </c>
       <c r="BQ35" s="11" t="n">
-        <v>63.077</v>
+        <v>22.42</v>
       </c>
       <c r="BR35" s="11" t="n">
-        <v>63.756</v>
+        <v>22.983</v>
       </c>
       <c r="BS35" s="11" t="n">
-        <v>62.852</v>
+        <v>22.773</v>
       </c>
       <c r="BT35" s="11" t="n">
-        <v>64.91200000000001</v>
+        <v>22.92</v>
       </c>
       <c r="BU35" s="11" t="n">
         <v>0</v>
       </c>
       <c r="BV35" s="11" t="n">
-        <v>-6.57</v>
+        <v>-5.1</v>
       </c>
       <c r="BW35" s="8" t="inlineStr">
         <is>
@@ -15228,7 +15284,7 @@
         </is>
       </c>
       <c r="BX35" s="11" t="n">
-        <v>-9.59</v>
+        <v>-9.279999999999999</v>
       </c>
       <c r="BY35" s="8" t="inlineStr">
         <is>
@@ -15236,7 +15292,7 @@
         </is>
       </c>
       <c r="BZ35" s="11" t="n">
-        <v>-8.289999999999999</v>
+        <v>-8.44</v>
       </c>
       <c r="CA35" s="8" t="inlineStr">
         <is>
@@ -15244,7 +15300,7 @@
         </is>
       </c>
       <c r="CB35" s="11" t="n">
-        <v>-11.2</v>
+        <v>-9.029999999999999</v>
       </c>
       <c r="CC35" s="20" t="inlineStr">
         <is>
@@ -15264,13 +15320,13 @@
         <v>5</v>
       </c>
       <c r="CH35" s="9" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="CI35" s="9" t="n">
         <v>0</v>
       </c>
       <c r="CJ35" s="9" t="n">
-        <v>-5</v>
+        <v>5</v>
       </c>
       <c r="CK35" s="9" t="n">
         <v>0</v>
@@ -15289,10 +15345,10 @@
         </is>
       </c>
       <c r="CO35" s="11" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="CP35" s="11" t="n">
-        <v>16.2</v>
+        <v>57.9</v>
       </c>
       <c r="CQ35" s="9" t="inlineStr">
         <is>
@@ -15303,16 +15359,16 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>SZ002202</t>
+          <t>SZ300442</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>金风科技</t>
+          <t>润泽科技</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>16.06</v>
+        <v>57.64</v>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
@@ -15320,31 +15376,31 @@
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>16.35</v>
+        <v>58.63</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>16.34</v>
+        <v>58.49</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>16.74</v>
+        <v>58.8</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>16.05</v>
+        <v>57.34</v>
       </c>
       <c r="I36" s="4" t="n">
-        <v>16.28</v>
+        <v>57.93</v>
       </c>
       <c r="J36" s="14" t="n">
-        <v>-1.77</v>
+        <v>-1.69</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>4.22</v>
+        <v>2.49</v>
       </c>
       <c r="L36" s="4" t="n">
-        <v>0.99</v>
+        <v>0.59</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>9.93</v>
+        <v>7.82</v>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
@@ -15352,10 +15408,10 @@
         </is>
       </c>
       <c r="O36" s="4" t="n">
-        <v>1.8</v>
+        <v>0.82</v>
       </c>
       <c r="P36" s="4" t="n">
-        <v>60.43</v>
+        <v>13.49</v>
       </c>
       <c r="Q36" s="4" t="n">
         <v>0</v>
@@ -15370,37 +15426,37 @@
         <v>0</v>
       </c>
       <c r="U36" s="14" t="n">
-        <v>-3.72</v>
+        <v>-7.67</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>3.88</v>
+        <v>5.8</v>
       </c>
       <c r="W36" s="4" t="n">
-        <v>16.36</v>
+        <v>59.57</v>
       </c>
       <c r="X36" s="4" t="n">
-        <v>16.34</v>
+        <v>58.49</v>
       </c>
       <c r="Y36" s="4" t="n">
-        <v>16.06</v>
+        <v>57.64</v>
       </c>
       <c r="Z36" s="4" t="n">
-        <v>17.99</v>
+        <v>63.46</v>
       </c>
       <c r="AA36" s="14" t="n">
-        <v>-10.73</v>
+        <v>-9.17</v>
       </c>
       <c r="AB36" s="4" t="n">
-        <v>15.93</v>
+        <v>55.92</v>
       </c>
       <c r="AC36" s="4" t="n">
-        <v>18.25</v>
+        <v>68.52</v>
       </c>
       <c r="AD36" s="4" t="n">
-        <v>15.93</v>
+        <v>55.92</v>
       </c>
       <c r="AE36" s="4" t="n">
-        <v>17.35</v>
+        <v>66.98999999999999</v>
       </c>
       <c r="AF36" s="2" t="inlineStr">
         <is>
@@ -15421,10 +15477,10 @@
         <v>0</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>5.19</v>
+        <v>4.26</v>
       </c>
       <c r="AK36" s="4" t="n">
-        <v>15.54</v>
+        <v>19.98</v>
       </c>
       <c r="AL36" s="8" t="inlineStr">
         <is>
@@ -15437,10 +15493,10 @@
         </is>
       </c>
       <c r="AN36" s="4" t="n">
-        <v>15.93</v>
+        <v>55.92</v>
       </c>
       <c r="AO36" s="4" t="n">
-        <v>0.8100000000000001</v>
+        <v>2.98</v>
       </c>
       <c r="AP36" s="8" t="inlineStr">
         <is>
@@ -15449,23 +15505,23 @@
       </c>
       <c r="AQ36" s="2" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>上升</t>
         </is>
       </c>
       <c r="AR36" s="4" t="n">
-        <v>0.876</v>
+        <v>0.82</v>
       </c>
       <c r="AS36" s="4" t="n">
-        <v>0.952</v>
+        <v>0.888</v>
       </c>
       <c r="AT36" s="4" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.976</v>
       </c>
       <c r="AU36" s="4" t="n">
-        <v>0.971</v>
+        <v>0.968</v>
       </c>
       <c r="AV36" s="4" t="n">
-        <v>0.876</v>
+        <v>0.82</v>
       </c>
       <c r="AW36" s="8" t="inlineStr">
         <is>
@@ -15476,14 +15532,14 @@
         <v>-5</v>
       </c>
       <c r="AY36" s="4" t="n">
-        <v>2.49</v>
+        <v>1.26</v>
       </c>
       <c r="AZ36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="BA36" s="2" t="inlineStr">
         <is>
-          <t>主板</t>
+          <t>科创/创业板</t>
         </is>
       </c>
       <c r="BB36" s="2" t="inlineStr">
@@ -15492,32 +15548,32 @@
         </is>
       </c>
       <c r="BC36" s="4" t="n">
-        <v>5.48</v>
-      </c>
-      <c r="BD36" s="8" t="inlineStr">
-        <is>
-          <t>极度超卖</t>
+        <v>43.99</v>
+      </c>
+      <c r="BD36" s="19" t="inlineStr">
+        <is>
+          <t>偏弱区</t>
         </is>
       </c>
       <c r="BE36" s="4" t="n">
-        <v>9.57</v>
+        <v>27.4</v>
       </c>
       <c r="BF36" s="4" t="n">
-        <v>12.3</v>
+        <v>42.62</v>
       </c>
       <c r="BG36" s="4" t="n">
-        <v>4.11</v>
-      </c>
-      <c r="BH36" s="8" t="inlineStr">
-        <is>
-          <t>低位钝化</t>
+        <v>-3.03</v>
+      </c>
+      <c r="BH36" s="19" t="inlineStr">
+        <is>
+          <t>偏空</t>
         </is>
       </c>
       <c r="BI36" s="4" t="n">
-        <v>-27.1</v>
+        <v>-25.29</v>
       </c>
       <c r="BJ36" s="4" t="n">
-        <v>30.26</v>
+        <v>42.39</v>
       </c>
       <c r="BK36" s="2" t="inlineStr">
         <is>
@@ -15537,49 +15593,49 @@
         </is>
       </c>
       <c r="BP36" s="4" t="n">
-        <v>16.68</v>
+        <v>61.696</v>
       </c>
       <c r="BQ36" s="4" t="n">
-        <v>16.933</v>
+        <v>63.077</v>
       </c>
       <c r="BR36" s="4" t="n">
-        <v>17.246</v>
+        <v>63.756</v>
       </c>
       <c r="BS36" s="4" t="n">
-        <v>17.762</v>
+        <v>62.852</v>
       </c>
       <c r="BT36" s="4" t="n">
-        <v>18.611</v>
+        <v>64.91200000000001</v>
       </c>
       <c r="BU36" s="4" t="n">
         <v>0</v>
       </c>
       <c r="BV36" s="4" t="n">
-        <v>-3.72</v>
+        <v>-6.57</v>
       </c>
       <c r="BW36" s="8" t="inlineStr">
         <is>
+          <t>极度超卖</t>
+        </is>
+      </c>
+      <c r="BX36" s="4" t="n">
+        <v>-9.59</v>
+      </c>
+      <c r="BY36" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
+        </is>
+      </c>
+      <c r="BZ36" s="4" t="n">
+        <v>-8.289999999999999</v>
+      </c>
+      <c r="CA36" s="8" t="inlineStr">
+        <is>
           <t>超卖偏弱</t>
         </is>
       </c>
-      <c r="BX36" s="4" t="n">
-        <v>-6.88</v>
-      </c>
-      <c r="BY36" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
-        </is>
-      </c>
-      <c r="BZ36" s="4" t="n">
-        <v>-9.58</v>
-      </c>
-      <c r="CA36" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
-        </is>
-      </c>
       <c r="CB36" s="4" t="n">
-        <v>-13.71</v>
+        <v>-11.2</v>
       </c>
       <c r="CC36" s="20" t="inlineStr">
         <is>
@@ -15590,7 +15646,7 @@
         <v>0</v>
       </c>
       <c r="CE36" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="CF36" s="2" t="n">
         <v>5</v>
@@ -15599,7 +15655,7 @@
         <v>5</v>
       </c>
       <c r="CH36" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="CI36" s="2" t="n">
         <v>0</v>
@@ -15611,7 +15667,7 @@
         <v>0</v>
       </c>
       <c r="CL36" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="CM36" s="18" t="inlineStr">
         <is>
@@ -15624,10 +15680,10 @@
         </is>
       </c>
       <c r="CO36" s="4" t="n">
-        <v>8.1</v>
+        <v>18.4</v>
       </c>
       <c r="CP36" s="4" t="n">
-        <v>29.7</v>
+        <v>15.8</v>
       </c>
       <c r="CQ36" s="2" t="inlineStr">
         <is>
@@ -15638,16 +15694,16 @@
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>SZ002245</t>
+          <t>SZ002202</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>蔚蓝锂芯</t>
+          <t>金风科技</t>
         </is>
       </c>
       <c r="C37" s="11" t="n">
-        <v>15.77</v>
+        <v>16.06</v>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
@@ -15655,31 +15711,31 @@
         </is>
       </c>
       <c r="E37" s="11" t="n">
-        <v>16.09</v>
+        <v>16.35</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>16</v>
+        <v>16.34</v>
       </c>
       <c r="G37" s="11" t="n">
-        <v>16.64</v>
+        <v>16.74</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>15.71</v>
+        <v>16.05</v>
       </c>
       <c r="I37" s="11" t="n">
-        <v>16.04</v>
+        <v>16.28</v>
       </c>
       <c r="J37" s="16" t="n">
-        <v>-1.99</v>
+        <v>-1.77</v>
       </c>
       <c r="K37" s="11" t="n">
-        <v>5.78</v>
+        <v>4.22</v>
       </c>
       <c r="L37" s="11" t="n">
-        <v>0.92</v>
+        <v>0.99</v>
       </c>
       <c r="M37" s="11" t="n">
-        <v>9.75</v>
+        <v>9.93</v>
       </c>
       <c r="N37" s="9" t="inlineStr">
         <is>
@@ -15687,10 +15743,10 @@
         </is>
       </c>
       <c r="O37" s="11" t="n">
-        <v>3.76</v>
+        <v>1.8</v>
       </c>
       <c r="P37" s="11" t="n">
-        <v>60.46</v>
+        <v>60.43</v>
       </c>
       <c r="Q37" s="11" t="n">
         <v>0</v>
@@ -15705,37 +15761,37 @@
         <v>0</v>
       </c>
       <c r="U37" s="16" t="n">
-        <v>-3.55</v>
+        <v>-3.72</v>
       </c>
       <c r="V37" s="11" t="n">
-        <v>5.62</v>
+        <v>3.88</v>
       </c>
       <c r="W37" s="11" t="n">
-        <v>16.07</v>
+        <v>16.36</v>
       </c>
       <c r="X37" s="11" t="n">
-        <v>16</v>
+        <v>16.34</v>
       </c>
       <c r="Y37" s="11" t="n">
-        <v>15.77</v>
+        <v>16.06</v>
       </c>
       <c r="Z37" s="11" t="n">
-        <v>17.14</v>
+        <v>17.99</v>
       </c>
       <c r="AA37" s="16" t="n">
-        <v>-7.99</v>
+        <v>-10.73</v>
       </c>
       <c r="AB37" s="11" t="n">
-        <v>15.45</v>
+        <v>15.93</v>
       </c>
       <c r="AC37" s="11" t="n">
-        <v>18.39</v>
+        <v>18.25</v>
       </c>
       <c r="AD37" s="11" t="n">
-        <v>15.45</v>
+        <v>15.93</v>
       </c>
       <c r="AE37" s="11" t="n">
-        <v>17.2</v>
+        <v>17.35</v>
       </c>
       <c r="AF37" s="9" t="inlineStr">
         <is>
@@ -15756,10 +15812,10 @@
         <v>0</v>
       </c>
       <c r="AJ37" s="11" t="n">
-        <v>3.12</v>
+        <v>5.19</v>
       </c>
       <c r="AK37" s="11" t="n">
-        <v>10.47</v>
+        <v>15.54</v>
       </c>
       <c r="AL37" s="8" t="inlineStr">
         <is>
@@ -15772,10 +15828,10 @@
         </is>
       </c>
       <c r="AN37" s="11" t="n">
-        <v>15.45</v>
+        <v>15.93</v>
       </c>
       <c r="AO37" s="11" t="n">
-        <v>2.03</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AP37" s="8" t="inlineStr">
         <is>
@@ -15788,19 +15844,19 @@
         </is>
       </c>
       <c r="AR37" s="11" t="n">
-        <v>0.909</v>
+        <v>0.876</v>
       </c>
       <c r="AS37" s="11" t="n">
-        <v>0.986</v>
+        <v>0.952</v>
       </c>
       <c r="AT37" s="11" t="n">
-        <v>0.952</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="AU37" s="11" t="n">
-        <v>0.923</v>
+        <v>0.971</v>
       </c>
       <c r="AV37" s="11" t="n">
-        <v>0.909</v>
+        <v>0.876</v>
       </c>
       <c r="AW37" s="8" t="inlineStr">
         <is>
@@ -15808,10 +15864,10 @@
         </is>
       </c>
       <c r="AX37" s="9" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="AY37" s="11" t="n">
-        <v>3.35</v>
+        <v>2.49</v>
       </c>
       <c r="AZ37" s="9" t="n">
         <v>0</v>
@@ -15827,7 +15883,7 @@
         </is>
       </c>
       <c r="BC37" s="11" t="n">
-        <v>19.55</v>
+        <v>5.48</v>
       </c>
       <c r="BD37" s="8" t="inlineStr">
         <is>
@@ -15835,13 +15891,13 @@
         </is>
       </c>
       <c r="BE37" s="11" t="n">
-        <v>14.59</v>
+        <v>9.57</v>
       </c>
       <c r="BF37" s="11" t="n">
-        <v>16.78</v>
+        <v>12.3</v>
       </c>
       <c r="BG37" s="11" t="n">
-        <v>10.21</v>
+        <v>4.11</v>
       </c>
       <c r="BH37" s="8" t="inlineStr">
         <is>
@@ -15849,10 +15905,10 @@
         </is>
       </c>
       <c r="BI37" s="11" t="n">
-        <v>-27.62</v>
+        <v>-27.1</v>
       </c>
       <c r="BJ37" s="11" t="n">
-        <v>42.35</v>
+        <v>30.26</v>
       </c>
       <c r="BK37" s="9" t="inlineStr">
         <is>
@@ -15872,63 +15928,63 @@
         </is>
       </c>
       <c r="BP37" s="11" t="n">
-        <v>16.114</v>
+        <v>16.68</v>
       </c>
       <c r="BQ37" s="11" t="n">
-        <v>16.224</v>
+        <v>16.933</v>
       </c>
       <c r="BR37" s="11" t="n">
-        <v>16.484</v>
+        <v>17.246</v>
       </c>
       <c r="BS37" s="11" t="n">
-        <v>17.241</v>
+        <v>17.762</v>
       </c>
       <c r="BT37" s="11" t="n">
-        <v>17.444</v>
+        <v>18.611</v>
       </c>
       <c r="BU37" s="11" t="n">
         <v>0</v>
       </c>
       <c r="BV37" s="11" t="n">
-        <v>-2.13</v>
-      </c>
-      <c r="BW37" s="20" t="inlineStr">
+        <v>-3.72</v>
+      </c>
+      <c r="BW37" s="8" t="inlineStr">
+        <is>
+          <t>超卖偏弱</t>
+        </is>
+      </c>
+      <c r="BX37" s="11" t="n">
+        <v>-6.88</v>
+      </c>
+      <c r="BY37" s="8" t="inlineStr">
+        <is>
+          <t>超卖偏弱</t>
+        </is>
+      </c>
+      <c r="BZ37" s="11" t="n">
+        <v>-9.58</v>
+      </c>
+      <c r="CA37" s="8" t="inlineStr">
+        <is>
+          <t>超卖偏弱</t>
+        </is>
+      </c>
+      <c r="CB37" s="11" t="n">
+        <v>-13.71</v>
+      </c>
+      <c r="CC37" s="20" t="inlineStr">
         <is>
           <t>中性区间</t>
         </is>
       </c>
-      <c r="BX37" s="11" t="n">
-        <v>-4.33</v>
-      </c>
-      <c r="BY37" s="20" t="inlineStr">
-        <is>
-          <t>中性区间</t>
-        </is>
-      </c>
-      <c r="BZ37" s="11" t="n">
-        <v>-8.529999999999999</v>
-      </c>
-      <c r="CA37" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
-        </is>
-      </c>
-      <c r="CB37" s="11" t="n">
-        <v>-9.6</v>
-      </c>
-      <c r="CC37" s="20" t="inlineStr">
-        <is>
-          <t>中性区间</t>
-        </is>
-      </c>
       <c r="CD37" s="9" t="n">
         <v>0</v>
       </c>
       <c r="CE37" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CF37" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CG37" s="9" t="n">
         <v>5</v>
@@ -15940,13 +15996,13 @@
         <v>0</v>
       </c>
       <c r="CJ37" s="9" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="CK37" s="9" t="n">
         <v>0</v>
       </c>
       <c r="CL37" s="9" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="CM37" s="18" t="inlineStr">
         <is>
@@ -15959,10 +16015,10 @@
         </is>
       </c>
       <c r="CO37" s="11" t="n">
-        <v>4.1</v>
+        <v>7.9</v>
       </c>
       <c r="CP37" s="11" t="n">
-        <v>37.8</v>
+        <v>28.9</v>
       </c>
       <c r="CQ37" s="9" t="inlineStr">
         <is>
@@ -15973,16 +16029,16 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>SZ000657</t>
+          <t>SZ002245</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>中钨高新</t>
+          <t>蔚蓝锂芯</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>48.34</v>
+        <v>15.77</v>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
@@ -15990,31 +16046,31 @@
         </is>
       </c>
       <c r="E38" s="4" t="n">
-        <v>51.13</v>
+        <v>16.09</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>50.9</v>
+        <v>16</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>50.9</v>
+        <v>16.64</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>48.24</v>
+        <v>15.71</v>
       </c>
       <c r="I38" s="4" t="n">
-        <v>49.16</v>
+        <v>16.04</v>
       </c>
       <c r="J38" s="14" t="n">
-        <v>-5.46</v>
+        <v>-1.99</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>5.2</v>
+        <v>5.78</v>
       </c>
       <c r="L38" s="4" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="M38" s="4" t="n">
-        <v>15.73</v>
+        <v>9.75</v>
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
@@ -16022,10 +16078,10 @@
         </is>
       </c>
       <c r="O38" s="4" t="n">
-        <v>2.2</v>
+        <v>3.76</v>
       </c>
       <c r="P38" s="4" t="n">
-        <v>31.98</v>
+        <v>60.46</v>
       </c>
       <c r="Q38" s="4" t="n">
         <v>0</v>
@@ -16040,37 +16096,37 @@
         <v>0</v>
       </c>
       <c r="U38" s="14" t="n">
-        <v>-6.77</v>
+        <v>-3.55</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>5.29</v>
+        <v>5.62</v>
       </c>
       <c r="W38" s="4" t="n">
-        <v>50.44</v>
+        <v>16.07</v>
       </c>
       <c r="X38" s="4" t="n">
-        <v>50.9</v>
+        <v>16</v>
       </c>
       <c r="Y38" s="4" t="n">
-        <v>48.34</v>
+        <v>15.77</v>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>58.7</v>
+        <v>17.14</v>
       </c>
       <c r="AA38" s="14" t="n">
-        <v>-17.65</v>
+        <v>-7.99</v>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>48.24</v>
+        <v>15.45</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>62.46</v>
+        <v>18.39</v>
       </c>
       <c r="AD38" s="4" t="n">
-        <v>48.24</v>
+        <v>15.45</v>
       </c>
       <c r="AE38" s="4" t="n">
-        <v>54.48</v>
+        <v>17.2</v>
       </c>
       <c r="AF38" s="2" t="inlineStr">
         <is>
@@ -16084,17 +16140,17 @@
       </c>
       <c r="AH38" s="2" t="inlineStr">
         <is>
-          <t>光头大阴</t>
+          <t>小阴线</t>
         </is>
       </c>
       <c r="AI38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>2.76</v>
+        <v>3.12</v>
       </c>
       <c r="AK38" s="4" t="n">
-        <v>19.07</v>
+        <v>10.47</v>
       </c>
       <c r="AL38" s="8" t="inlineStr">
         <is>
@@ -16107,10 +16163,10 @@
         </is>
       </c>
       <c r="AN38" s="4" t="n">
-        <v>48.24</v>
+        <v>15.45</v>
       </c>
       <c r="AO38" s="4" t="n">
-        <v>0.21</v>
+        <v>2.03</v>
       </c>
       <c r="AP38" s="8" t="inlineStr">
         <is>
@@ -16123,19 +16179,19 @@
         </is>
       </c>
       <c r="AR38" s="4" t="n">
-        <v>0.763</v>
+        <v>0.909</v>
       </c>
       <c r="AS38" s="4" t="n">
-        <v>0.912</v>
+        <v>0.986</v>
       </c>
       <c r="AT38" s="4" t="n">
-        <v>0.846</v>
+        <v>0.952</v>
       </c>
       <c r="AU38" s="4" t="n">
-        <v>0.86</v>
+        <v>0.923</v>
       </c>
       <c r="AV38" s="4" t="n">
-        <v>0.763</v>
+        <v>0.909</v>
       </c>
       <c r="AW38" s="8" t="inlineStr">
         <is>
@@ -16143,10 +16199,10 @@
         </is>
       </c>
       <c r="AX38" s="2" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="AY38" s="4" t="n">
-        <v>3.47</v>
+        <v>3.35</v>
       </c>
       <c r="AZ38" s="2" t="n">
         <v>0</v>
@@ -16162,32 +16218,32 @@
         </is>
       </c>
       <c r="BC38" s="4" t="n">
-        <v>22.3</v>
+        <v>19.55</v>
       </c>
       <c r="BD38" s="8" t="inlineStr">
         <is>
-          <t>超卖区</t>
+          <t>极度超卖</t>
         </is>
       </c>
       <c r="BE38" s="4" t="n">
-        <v>9.050000000000001</v>
+        <v>14.59</v>
       </c>
       <c r="BF38" s="4" t="n">
-        <v>15.83</v>
+        <v>16.78</v>
       </c>
       <c r="BG38" s="4" t="n">
-        <v>-4.5</v>
+        <v>10.21</v>
       </c>
       <c r="BH38" s="8" t="inlineStr">
         <is>
-          <t>极度超卖</t>
+          <t>低位钝化</t>
         </is>
       </c>
       <c r="BI38" s="4" t="n">
-        <v>-35.83</v>
+        <v>-27.62</v>
       </c>
       <c r="BJ38" s="4" t="n">
-        <v>43.32</v>
+        <v>42.35</v>
       </c>
       <c r="BK38" s="2" t="inlineStr">
         <is>
@@ -16207,53 +16263,53 @@
         </is>
       </c>
       <c r="BP38" s="4" t="n">
-        <v>51.55</v>
+        <v>16.114</v>
       </c>
       <c r="BQ38" s="4" t="n">
-        <v>52.597</v>
+        <v>16.224</v>
       </c>
       <c r="BR38" s="4" t="n">
-        <v>54.809</v>
+        <v>16.484</v>
       </c>
       <c r="BS38" s="4" t="n">
-        <v>57.624</v>
+        <v>17.241</v>
       </c>
       <c r="BT38" s="4" t="n">
-        <v>60.914</v>
+        <v>17.444</v>
       </c>
       <c r="BU38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="BV38" s="4" t="n">
-        <v>-6.23</v>
-      </c>
-      <c r="BW38" s="8" t="inlineStr">
-        <is>
-          <t>极度超卖</t>
+        <v>-2.13</v>
+      </c>
+      <c r="BW38" s="20" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="BX38" s="4" t="n">
-        <v>-11.8</v>
-      </c>
-      <c r="BY38" s="8" t="inlineStr">
-        <is>
-          <t>极度超卖</t>
+        <v>-4.33</v>
+      </c>
+      <c r="BY38" s="20" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="BZ38" s="4" t="n">
-        <v>-16.11</v>
+        <v>-8.529999999999999</v>
       </c>
       <c r="CA38" s="8" t="inlineStr">
         <is>
-          <t>极度超卖</t>
+          <t>超卖偏弱</t>
         </is>
       </c>
       <c r="CB38" s="4" t="n">
-        <v>-20.64</v>
-      </c>
-      <c r="CC38" s="8" t="inlineStr">
-        <is>
-          <t>极度超卖</t>
+        <v>-9.6</v>
+      </c>
+      <c r="CC38" s="20" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="CD38" s="2" t="n">
@@ -16263,7 +16319,7 @@
         <v>0</v>
       </c>
       <c r="CF38" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="CG38" s="2" t="n">
         <v>5</v>
@@ -16275,7 +16331,7 @@
         <v>0</v>
       </c>
       <c r="CJ38" s="2" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="CK38" s="2" t="n">
         <v>0</v>
@@ -16294,19 +16350,354 @@
         </is>
       </c>
       <c r="CO38" s="4" t="n">
-        <v>4.1</v>
+        <v>3.9</v>
       </c>
       <c r="CP38" s="4" t="n">
-        <v>5.4</v>
+        <v>39.5</v>
       </c>
       <c r="CQ38" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>SZ000657</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>中钨高新</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="n">
+        <v>48.34</v>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>弱势</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="n">
+        <v>51.13</v>
+      </c>
+      <c r="F39" s="11" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="G39" s="11" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="H39" s="11" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="I39" s="11" t="n">
+        <v>49.16</v>
+      </c>
+      <c r="J39" s="16" t="n">
+        <v>-5.46</v>
+      </c>
+      <c r="K39" s="11" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="L39" s="11" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="M39" s="11" t="n">
+        <v>15.73</v>
+      </c>
+      <c r="N39" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="O39" s="11" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="P39" s="11" t="n">
+        <v>31.98</v>
+      </c>
+      <c r="Q39" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U39" s="16" t="n">
+        <v>-6.77</v>
+      </c>
+      <c r="V39" s="11" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="W39" s="11" t="n">
+        <v>50.44</v>
+      </c>
+      <c r="X39" s="11" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="Y39" s="11" t="n">
+        <v>48.34</v>
+      </c>
+      <c r="Z39" s="11" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="AA39" s="16" t="n">
+        <v>-17.65</v>
+      </c>
+      <c r="AB39" s="11" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="AC39" s="11" t="n">
+        <v>62.46</v>
+      </c>
+      <c r="AD39" s="11" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="AE39" s="11" t="n">
+        <v>54.48</v>
+      </c>
+      <c r="AF39" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AG39" s="9" t="inlineStr">
+        <is>
+          <t>无明显形态</t>
+        </is>
+      </c>
+      <c r="AH39" s="9" t="inlineStr">
+        <is>
+          <t>光头大阴</t>
+        </is>
+      </c>
+      <c r="AI39" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ39" s="11" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="AK39" s="11" t="n">
+        <v>19.07</v>
+      </c>
+      <c r="AL39" s="8" t="inlineStr">
+        <is>
+          <t>无趋势</t>
+        </is>
+      </c>
+      <c r="AM39" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AN39" s="11" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="AO39" s="11" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AP39" s="8" t="inlineStr">
+        <is>
+          <t>极低波动盘整</t>
+        </is>
+      </c>
+      <c r="AQ39" s="9" t="inlineStr">
+        <is>
+          <t>下降</t>
+        </is>
+      </c>
+      <c r="AR39" s="11" t="n">
+        <v>0.763</v>
+      </c>
+      <c r="AS39" s="11" t="n">
+        <v>0.912</v>
+      </c>
+      <c r="AT39" s="11" t="n">
+        <v>0.846</v>
+      </c>
+      <c r="AU39" s="11" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AV39" s="11" t="n">
+        <v>0.763</v>
+      </c>
+      <c r="AW39" s="8" t="inlineStr">
+        <is>
+          <t>总体偏弱</t>
+        </is>
+      </c>
+      <c r="AX39" s="9" t="n">
+        <v>-5</v>
+      </c>
+      <c r="AY39" s="11" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="AZ39" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA39" s="9" t="inlineStr">
+        <is>
+          <t>主板</t>
+        </is>
+      </c>
+      <c r="BB39" s="9" t="inlineStr">
+        <is>
+          <t>沪深300</t>
+        </is>
+      </c>
+      <c r="BC39" s="11" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="BD39" s="8" t="inlineStr">
+        <is>
+          <t>超卖区</t>
+        </is>
+      </c>
+      <c r="BE39" s="11" t="n">
+        <v>9.050000000000001</v>
+      </c>
+      <c r="BF39" s="11" t="n">
+        <v>15.83</v>
+      </c>
+      <c r="BG39" s="11" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="BH39" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
+        </is>
+      </c>
+      <c r="BI39" s="11" t="n">
+        <v>-35.83</v>
+      </c>
+      <c r="BJ39" s="11" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="BK39" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="BL39" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="BM39" s="9" t="inlineStr"/>
+      <c r="BN39" s="9" t="inlineStr"/>
+      <c r="BO39" s="7" t="inlineStr">
+        <is>
+          <t>深回撤|弱市</t>
+        </is>
+      </c>
+      <c r="BP39" s="11" t="n">
+        <v>51.55</v>
+      </c>
+      <c r="BQ39" s="11" t="n">
+        <v>52.597</v>
+      </c>
+      <c r="BR39" s="11" t="n">
+        <v>54.809</v>
+      </c>
+      <c r="BS39" s="11" t="n">
+        <v>57.624</v>
+      </c>
+      <c r="BT39" s="11" t="n">
+        <v>60.914</v>
+      </c>
+      <c r="BU39" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV39" s="11" t="n">
+        <v>-6.23</v>
+      </c>
+      <c r="BW39" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
+        </is>
+      </c>
+      <c r="BX39" s="11" t="n">
+        <v>-11.8</v>
+      </c>
+      <c r="BY39" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
+        </is>
+      </c>
+      <c r="BZ39" s="11" t="n">
+        <v>-16.11</v>
+      </c>
+      <c r="CA39" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
+        </is>
+      </c>
+      <c r="CB39" s="11" t="n">
+        <v>-20.64</v>
+      </c>
+      <c r="CC39" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
+        </is>
+      </c>
+      <c r="CD39" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE39" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF39" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="CG39" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="CH39" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="CI39" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ39" s="9" t="n">
+        <v>-5</v>
+      </c>
+      <c r="CK39" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL39" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="CM39" s="18" t="inlineStr">
+        <is>
+          <t>D 级 (风险)</t>
+        </is>
+      </c>
+      <c r="CN39" s="9" t="inlineStr">
+        <is>
+          <t>排除/止损 | 弱市慎加仓</t>
+        </is>
+      </c>
+      <c r="CO39" s="11" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="CP39" s="11" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="CQ39" s="9" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="CL2:CL38">
+  <conditionalFormatting sqref="CL2:CL39">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="15"/>
@@ -16318,7 +16709,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="CO2:CO38">
+  <conditionalFormatting sqref="CO2:CO39">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -16330,7 +16721,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AR2:AR38">
+  <conditionalFormatting sqref="AR2:AR39">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -16342,7 +16733,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AS2:AS38">
+  <conditionalFormatting sqref="AS2:AS39">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -16354,7 +16745,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AT2:AT38">
+  <conditionalFormatting sqref="AT2:AT39">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -16366,7 +16757,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AU2:AU38">
+  <conditionalFormatting sqref="AU2:AU39">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -16378,7 +16769,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AV2:AV38">
+  <conditionalFormatting sqref="AV2:AV39">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -16390,7 +16781,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK2:AK38">
+  <conditionalFormatting sqref="AK2:AK39">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="num" val="15"/>
@@ -17543,7 +17934,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -17583,7 +17974,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -17637,7 +18028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -17657,13 +18048,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>SZ300831: SZ300831 数据获取失败（AkShare+Baostock均失败）</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto stock scan 2026-10-13 15:28 UTC
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -2967,12 +2967,12 @@
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="11.23529411764706" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="15.875" customWidth="1" min="24" max="24"/>
+    <col width="26.5" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -3285,46 +3285,46 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
+        <v>24345.22</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>24271.2</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>24211.35</v>
-      </c>
       <c r="E4" s="4" t="n">
-        <v>24434.93</v>
+        <v>24172.09</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>24455.95</v>
+        <v>24345.22</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>24193.3</v>
+        <v>23987.77</v>
       </c>
       <c r="H4" s="17" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1.08</v>
+        <v>1.47</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>24135.88</v>
+        <v>24148.812</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>24247.138</v>
+        <v>24217.409</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>24773.278</v>
+        <v>24732.552</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>25151.488</v>
+        <v>25138.191</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>25062.025</v>
+        <v>25044.173</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>23737.14</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>24767.22</v>
+        <v>24648.64</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>23737.14</v>
@@ -3334,7 +3334,7 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是（最近金叉）</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
@@ -3344,11 +3344,11 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>小阴线</t>
+          <t>中阳线</t>
         </is>
       </c>
       <c r="V4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W4" s="8" t="inlineStr">
         <is>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>跌破MA60 | 近期连阳</t>
+          <t>跌破MA60 | 近期连阳 | 是（最近金叉）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto stock scan 2026-10-21 09:06 UTC
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -185,7 +185,7 @@
     <xf numFmtId="2" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -197,7 +197,7 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -578,7 +578,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16.5" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
@@ -659,22 +659,22 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SZ300831</t>
+          <t>SZ000555</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>派瑞股份</t>
+          <t>神州信息</t>
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>12.11</v>
+        <v>10.24</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>1.17</v>
+        <v>3.23</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
@@ -695,7 +695,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>深回撤|弱市</t>
+          <t>弱市</t>
         </is>
       </c>
       <c r="L2" s="4" t="n">
@@ -715,22 +715,22 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>SZ000582</t>
+          <t>SZ002241</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>北部湾港</t>
+          <t>歌尔股份</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>9.109999999999999</v>
+        <v>21.04</v>
       </c>
       <c r="D3" s="12" t="n">
-        <v>1.67</v>
+        <v>-2.23</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
@@ -744,10 +744,14 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>MACD金叉</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="inlineStr"/>
+          <t>超跌蓄势</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>超跌蓄势</t>
+        </is>
+      </c>
       <c r="J3" s="9" t="inlineStr">
         <is>
           <t>否</t>
@@ -755,11 +759,11 @@
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>深回撤|弱市</t>
+          <t>弱市</t>
         </is>
       </c>
       <c r="L3" s="11" t="n">
-        <v>80</v>
+        <v>85.7</v>
       </c>
       <c r="M3" s="8" t="inlineStr">
         <is>
@@ -775,22 +779,22 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>SZ002028</t>
+          <t>SZ002271</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>思源电气</t>
+          <t>东方雨虹</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>112.59</v>
-      </c>
-      <c r="D4" s="13" t="n">
-        <v>-10</v>
+        <v>10.71</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>0.66</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
@@ -802,11 +806,7 @@
           <t>排除/止损 | 弱市慎加仓</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>MACD金叉</t>
-        </is>
-      </c>
+      <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -815,11 +815,11 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>深回撤|弱市</t>
+          <t>弱市</t>
         </is>
       </c>
       <c r="L4" s="4" t="n">
-        <v>50</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="M4" s="8" t="inlineStr">
         <is>
@@ -835,19 +835,19 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>SZ002240</t>
+          <t>SZ002460</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>盛新锂能</t>
+          <t>赣锋锂业</t>
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>21.5</v>
+        <v>37.8</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>0.75</v>
+        <v>-1.12</v>
       </c>
       <c r="E5" s="9" t="n">
         <v>25</v>
@@ -891,22 +891,22 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SZ002223</t>
+          <t>SZ002466</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>鱼跃医疗</t>
+          <t>天齐锂业</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>25.66</v>
-      </c>
-      <c r="D6" s="13" t="n">
-        <v>-0.93</v>
+        <v>36.5</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0.19</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
@@ -927,25 +927,137 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
+          <t>深回撤|弱市</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>弱势</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>SZ002245</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>蔚蓝锂芯</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>12.87</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>-10</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>D 级 (风险)</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>排除/止损 | 弱市慎加仓</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr"/>
+      <c r="I7" s="9" t="inlineStr"/>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>深回撤|止损过宽|弱市</t>
+        </is>
+      </c>
+      <c r="L7" s="11" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>弱势</t>
+        </is>
+      </c>
+      <c r="N7" s="9" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SZ002223</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>鱼跃医疗</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>25.66</v>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>-0.93</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>D 级 (风险)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>排除/止损 | 弱市慎加仓</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
           <t>弱市</t>
         </is>
       </c>
-      <c r="L6" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="M6" s="8" t="inlineStr">
+      <c r="L8" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="M8" s="8" t="inlineStr">
         <is>
           <t>弱势</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E6">
+  <conditionalFormatting sqref="E2:E8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="15"/>
@@ -957,7 +1069,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L6">
+  <conditionalFormatting sqref="L2:L8">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -1005,7 +1117,7 @@
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="19.625" customWidth="1" min="24" max="24"/>
+    <col width="26.5" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1142,40 +1254,40 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
+        <v>3735.37</v>
+      </c>
+      <c r="D2" s="4" t="n">
         <v>3730.92</v>
       </c>
-      <c r="D2" s="4" t="n">
-        <v>3716.28</v>
-      </c>
       <c r="E2" s="4" t="n">
-        <v>3694.12</v>
+        <v>3718.44</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>3743.8</v>
+        <v>3740.07</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3692.29</v>
+        <v>3702.44</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.39</v>
+        <v>0.12</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>1.39</v>
+        <v>1.01</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>3744.554</v>
+        <v>3731.455</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>3781.835</v>
+        <v>3772.327</v>
       </c>
       <c r="L2" s="4" t="n">
-        <v>3874.155</v>
+        <v>3865.79</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>3881.693</v>
+        <v>3880.678</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>3978.735</v>
+        <v>3975.821</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>3674.82</v>
@@ -1187,7 +1299,7 @@
         <v>3674.82</v>
       </c>
       <c r="R2" s="4" t="n">
-        <v>3822.1</v>
+        <v>3811.81</v>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
@@ -1201,7 +1313,7 @@
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>看涨吞没</t>
+          <t>小阳线</t>
         </is>
       </c>
       <c r="V2" s="2" t="n">
@@ -1230,40 +1342,40 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
+        <v>11801.29</v>
+      </c>
+      <c r="D3" s="11" t="n">
         <v>11817.42</v>
       </c>
-      <c r="D3" s="11" t="n">
-        <v>11802.46</v>
-      </c>
       <c r="E3" s="11" t="n">
-        <v>11743.22</v>
+        <v>11774.39</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>11884.16</v>
+        <v>11938</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>11667.18</v>
+        <v>11691.41</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>0.13</v>
+        <v>-0.14</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>1.84</v>
+        <v>2.09</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>11980.192</v>
+        <v>11869.71</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>12333.815</v>
+        <v>12223.749</v>
       </c>
       <c r="L3" s="11" t="n">
-        <v>13157.105</v>
+        <v>13083.315</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>13582.165</v>
+        <v>13552.016</v>
       </c>
       <c r="N3" s="11" t="n">
-        <v>14508.441</v>
+        <v>14481.933</v>
       </c>
       <c r="O3" s="11" t="n">
         <v>11667.18</v>
@@ -1275,7 +1387,7 @@
         <v>11667.18</v>
       </c>
       <c r="R3" s="11" t="n">
-        <v>12486.21</v>
+        <v>12383.62</v>
       </c>
       <c r="S3" s="9" t="inlineStr">
         <is>
@@ -1318,40 +1430,40 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
+        <v>23867.74</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>24186.83</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>24062.72</v>
-      </c>
       <c r="E4" s="4" t="n">
-        <v>24321.45</v>
+        <v>23990.05</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>24392.3</v>
+        <v>24035</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>24087.23</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>0.52</v>
+        <v>23846.99</v>
+      </c>
+      <c r="H4" s="13" t="n">
+        <v>-1.32</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1.27</v>
+        <v>0.78</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>24236.028</v>
+        <v>24155.336</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>24162.868</v>
+        <v>24145.608</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>24622.868</v>
+        <v>24563.43</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>25093.657</v>
+        <v>25075.398</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>24998.4</v>
+        <v>24981.251</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>23737.14</v>
@@ -1360,7 +1472,7 @@
         <v>24524.63</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>23945.84</v>
+        <v>23846.99</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>24524.63</v>
@@ -1390,7 +1502,7 @@
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>跌破MA60 | 是（最近金叉）</t>
+          <t>跌破MA60 | 是（最近金叉） | 日内偏弱</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ6"/>
+  <dimension ref="A1:CQ8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1439,7 +1551,7 @@
     <col width="12" customWidth="1" min="29" max="29"/>
     <col width="12" customWidth="1" min="30" max="30"/>
     <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="11.23529411764706" customWidth="1" min="32" max="32"/>
+    <col width="11" customWidth="1" min="32" max="32"/>
     <col width="14" customWidth="1" min="33" max="33"/>
     <col width="14" customWidth="1" min="34" max="34"/>
     <col width="11" customWidth="1" min="35" max="35"/>
@@ -1449,14 +1561,14 @@
     <col width="12" customWidth="1" min="39" max="39"/>
     <col width="11" customWidth="1" min="40" max="40"/>
     <col width="11" customWidth="1" min="41" max="41"/>
-    <col width="14" customWidth="1" min="42" max="42"/>
+    <col width="14.625" customWidth="1" min="42" max="42"/>
     <col width="14" customWidth="1" min="43" max="43"/>
     <col width="11" customWidth="1" min="44" max="44"/>
     <col width="11" customWidth="1" min="45" max="45"/>
     <col width="11" customWidth="1" min="46" max="46"/>
     <col width="11" customWidth="1" min="47" max="47"/>
     <col width="11" customWidth="1" min="48" max="48"/>
-    <col width="14" customWidth="1" min="49" max="49"/>
+    <col width="15.25" customWidth="1" min="49" max="49"/>
     <col width="11" customWidth="1" min="50" max="50"/>
     <col width="11.23529411764706" customWidth="1" min="51" max="51"/>
     <col width="11" customWidth="1" min="52" max="52"/>
@@ -1474,7 +1586,7 @@
     <col width="11" customWidth="1" min="64" max="64"/>
     <col width="14" customWidth="1" min="65" max="65"/>
     <col width="11" customWidth="1" min="66" max="66"/>
-    <col width="14" customWidth="1" min="67" max="67"/>
+    <col width="16.5" customWidth="1" min="67" max="67"/>
     <col width="11" customWidth="1" min="68" max="68"/>
     <col width="11" customWidth="1" min="69" max="69"/>
     <col width="11" customWidth="1" min="70" max="70"/>
@@ -1985,16 +2097,16 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SZ300831</t>
+          <t>SZ000555</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>派瑞股份</t>
+          <t>神州信息</t>
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>12.11</v>
+        <v>10.24</v>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
@@ -2002,31 +2114,31 @@
         </is>
       </c>
       <c r="E2" s="4" t="n">
-        <v>11.97</v>
+        <v>9.92</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>11.96</v>
+        <v>9.91</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>12.28</v>
+        <v>10.24</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>11.95</v>
+        <v>9.84</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>12.11</v>
+        <v>10.11</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>1.17</v>
+        <v>3.23</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>2.76</v>
+        <v>4.03</v>
       </c>
       <c r="L2" s="4" t="n">
-        <v>0.71</v>
+        <v>1.23</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>0</v>
+        <v>1.58</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -2034,10 +2146,10 @@
         </is>
       </c>
       <c r="O2" s="4" t="n">
-        <v>1.09</v>
+        <v>1.6</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>0.02</v>
+        <v>15.6</v>
       </c>
       <c r="Q2" s="4" t="n">
         <v>0</v>
@@ -2052,37 +2164,37 @@
         <v>1</v>
       </c>
       <c r="U2" s="5" t="n">
-        <v>0.58</v>
+        <v>3.23</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>3.09</v>
+        <v>3.73</v>
       </c>
       <c r="W2" s="4" t="n">
-        <v>12.04</v>
+        <v>10.03</v>
       </c>
       <c r="X2" s="4" t="n">
-        <v>11.96</v>
+        <v>9.91</v>
       </c>
       <c r="Y2" s="4" t="n">
-        <v>12.11</v>
+        <v>10.24</v>
       </c>
       <c r="Z2" s="4" t="n">
-        <v>13.37</v>
+        <v>10.27</v>
       </c>
       <c r="AA2" s="13" t="n">
-        <v>-9.42</v>
+        <v>-0.29</v>
       </c>
       <c r="AB2" s="4" t="n">
-        <v>11.7</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="AC2" s="4" t="n">
-        <v>13.53</v>
+        <v>10.43</v>
       </c>
       <c r="AD2" s="4" t="n">
-        <v>11.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="AE2" s="4" t="n">
-        <v>12.86</v>
+        <v>10.37</v>
       </c>
       <c r="AF2" s="2" t="inlineStr">
         <is>
@@ -2091,26 +2203,26 @@
       </c>
       <c r="AG2" s="2" t="inlineStr">
         <is>
-          <t>无明显形态</t>
+          <t>站上 MA20</t>
         </is>
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>看涨吞没</t>
+          <t>中阳线</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>2.54</v>
+        <v>4.46</v>
       </c>
       <c r="AK2" s="4" t="n">
-        <v>36.05</v>
-      </c>
-      <c r="AL2" s="14" t="inlineStr">
-        <is>
-          <t>强趋势</t>
+        <v>12.41</v>
+      </c>
+      <c r="AL2" s="8" t="inlineStr">
+        <is>
+          <t>无趋势</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
@@ -2119,53 +2231,53 @@
         </is>
       </c>
       <c r="AN2" s="4" t="n">
-        <v>11.7</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="AO2" s="4" t="n">
-        <v>3.39</v>
-      </c>
-      <c r="AP2" s="15" t="inlineStr">
-        <is>
-          <t>低波动平稳期</t>
+        <v>5.96</v>
+      </c>
+      <c r="AP2" s="14" t="inlineStr">
+        <is>
+          <t>健康趋势行情</t>
         </is>
       </c>
       <c r="AQ2" s="2" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>上升</t>
         </is>
       </c>
       <c r="AR2" s="4" t="n">
-        <v>1.003</v>
+        <v>1.114</v>
       </c>
       <c r="AS2" s="4" t="n">
-        <v>0.956</v>
+        <v>1.022</v>
       </c>
       <c r="AT2" s="4" t="n">
-        <v>0.93</v>
+        <v>1.067</v>
       </c>
       <c r="AU2" s="4" t="n">
-        <v>0.918</v>
+        <v>1.053</v>
       </c>
       <c r="AV2" s="4" t="n">
-        <v>1.003</v>
-      </c>
-      <c r="AW2" s="15" t="inlineStr">
-        <is>
-          <t>强弱不明，震荡</t>
+        <v>1.114</v>
+      </c>
+      <c r="AW2" s="14" t="inlineStr">
+        <is>
+          <t>总体偏强</t>
         </is>
       </c>
       <c r="AX2" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="AY2" s="4" t="n">
-        <v>1.63</v>
+        <v>1.84</v>
       </c>
       <c r="AZ2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="BA2" s="2" t="inlineStr">
         <is>
-          <t>科创/创业板</t>
+          <t>主板</t>
         </is>
       </c>
       <c r="BB2" s="2" t="inlineStr">
@@ -2174,32 +2286,32 @@
         </is>
       </c>
       <c r="BC2" s="4" t="n">
-        <v>9.16</v>
-      </c>
-      <c r="BD2" s="8" t="inlineStr">
-        <is>
-          <t>极度超卖</t>
+        <v>45.79</v>
+      </c>
+      <c r="BD2" s="15" t="inlineStr">
+        <is>
+          <t>偏弱区</t>
         </is>
       </c>
       <c r="BE2" s="4" t="n">
-        <v>15.38</v>
+        <v>51.47</v>
       </c>
       <c r="BF2" s="4" t="n">
-        <v>12.7</v>
+        <v>43.57</v>
       </c>
       <c r="BG2" s="4" t="n">
-        <v>20.72</v>
-      </c>
-      <c r="BH2" s="8" t="inlineStr">
-        <is>
-          <t>低位钝化</t>
+        <v>67.26000000000001</v>
+      </c>
+      <c r="BH2" s="14" t="inlineStr">
+        <is>
+          <t>偏多</t>
         </is>
       </c>
       <c r="BI2" s="4" t="n">
-        <v>-26.52</v>
+        <v>-13.16</v>
       </c>
       <c r="BJ2" s="4" t="n">
-        <v>23.69</v>
+        <v>47.49</v>
       </c>
       <c r="BK2" s="2" t="inlineStr">
         <is>
@@ -2215,29 +2327,29 @@
       <c r="BN2" s="2" t="inlineStr"/>
       <c r="BO2" s="7" t="inlineStr">
         <is>
-          <t>深回撤|弱市</t>
+          <t>弱市</t>
         </is>
       </c>
       <c r="BP2" s="4" t="n">
-        <v>12.1</v>
+        <v>10.032</v>
       </c>
       <c r="BQ2" s="4" t="n">
-        <v>12.31</v>
+        <v>10.12</v>
       </c>
       <c r="BR2" s="4" t="n">
-        <v>12.553</v>
+        <v>10.109</v>
       </c>
       <c r="BS2" s="4" t="n">
-        <v>13.296</v>
+        <v>10.223</v>
       </c>
       <c r="BT2" s="4" t="n">
-        <v>14.322</v>
+        <v>10.581</v>
       </c>
       <c r="BU2" s="4" t="n">
         <v>0</v>
       </c>
       <c r="BV2" s="4" t="n">
-        <v>0.08</v>
+        <v>2.07</v>
       </c>
       <c r="BW2" s="14" t="inlineStr">
         <is>
@@ -2245,7 +2357,7 @@
         </is>
       </c>
       <c r="BX2" s="4" t="n">
-        <v>-3.53</v>
+        <v>1.3</v>
       </c>
       <c r="BY2" s="14" t="inlineStr">
         <is>
@@ -2253,47 +2365,47 @@
         </is>
       </c>
       <c r="BZ2" s="4" t="n">
-        <v>-8.92</v>
-      </c>
-      <c r="CA2" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
+        <v>0.16</v>
+      </c>
+      <c r="CA2" s="14" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="CB2" s="4" t="n">
-        <v>-15.44</v>
-      </c>
-      <c r="CC2" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
+        <v>-3.22</v>
+      </c>
+      <c r="CC2" s="14" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="CD2" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="CE2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="CF2" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="CG2" s="2" t="n">
         <v>5</v>
       </c>
       <c r="CH2" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="CI2" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="CJ2" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="CK2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="CL2" s="2" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="CM2" s="6" t="inlineStr">
         <is>
@@ -2309,7 +2421,7 @@
         <v>100</v>
       </c>
       <c r="CP2" s="4" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="CQ2" s="2" t="inlineStr">
         <is>
@@ -2320,16 +2432,16 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>SZ000582</t>
+          <t>SZ002241</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>北部湾港</t>
+          <t>歌尔股份</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>9.109999999999999</v>
+        <v>21.04</v>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
@@ -2337,31 +2449,31 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>8.960000000000001</v>
+        <v>21.52</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>8.960000000000001</v>
+        <v>21.43</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>9.119999999999999</v>
+        <v>21.44</v>
       </c>
       <c r="H3" s="11" t="n">
-        <v>8.880000000000001</v>
+        <v>21</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>9.039999999999999</v>
+        <v>21.16</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>1.67</v>
+        <v>-2.23</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>2.68</v>
+        <v>2.04</v>
       </c>
       <c r="L3" s="11" t="n">
-        <v>0.82</v>
+        <v>1.03</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>0.03</v>
+        <v>0.12</v>
       </c>
       <c r="N3" s="9" t="inlineStr">
         <is>
@@ -2369,10 +2481,10 @@
         </is>
       </c>
       <c r="O3" s="11" t="n">
-        <v>1.47</v>
+        <v>1.85</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.32</v>
+        <v>0.58</v>
       </c>
       <c r="Q3" s="11" t="n">
         <v>0</v>
@@ -2384,68 +2496,68 @@
         <v>0</v>
       </c>
       <c r="T3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="16" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="V3" s="11" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="W3" s="11" t="n">
+        <v>20.89</v>
+      </c>
+      <c r="X3" s="11" t="n">
+        <v>21.43</v>
+      </c>
+      <c r="Y3" s="11" t="n">
+        <v>21.04</v>
+      </c>
+      <c r="Z3" s="11" t="n">
+        <v>22.57</v>
+      </c>
+      <c r="AA3" s="12" t="n">
+        <v>-6.78</v>
+      </c>
+      <c r="AB3" s="11" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="AC3" s="11" t="n">
+        <v>23.03</v>
+      </c>
+      <c r="AD3" s="11" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="AE3" s="11" t="n">
+        <v>21.58</v>
+      </c>
+      <c r="AF3" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AG3" s="9" t="inlineStr">
+        <is>
+          <t>无明显形态</t>
+        </is>
+      </c>
+      <c r="AH3" s="9" t="inlineStr">
+        <is>
+          <t>看跌孕线</t>
+        </is>
+      </c>
+      <c r="AI3" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="U3" s="12" t="n">
-        <v>1.67</v>
-      </c>
-      <c r="V3" s="11" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="W3" s="11" t="n">
-        <v>9.01</v>
-      </c>
-      <c r="X3" s="11" t="n">
-        <v>8.960000000000001</v>
-      </c>
-      <c r="Y3" s="11" t="n">
-        <v>9.109999999999999</v>
-      </c>
-      <c r="Z3" s="11" t="n">
-        <v>9.789999999999999</v>
-      </c>
-      <c r="AA3" s="16" t="n">
-        <v>-6.95</v>
-      </c>
-      <c r="AB3" s="11" t="n">
-        <v>8.720000000000001</v>
-      </c>
-      <c r="AC3" s="11" t="n">
-        <v>9.869999999999999</v>
-      </c>
-      <c r="AD3" s="11" t="n">
-        <v>8.779999999999999</v>
-      </c>
-      <c r="AE3" s="11" t="n">
-        <v>9.59</v>
-      </c>
-      <c r="AF3" s="9" t="inlineStr">
-        <is>
-          <t>是（最近金叉）</t>
-        </is>
-      </c>
-      <c r="AG3" s="9" t="inlineStr">
-        <is>
-          <t>无明显形态</t>
-        </is>
-      </c>
-      <c r="AH3" s="9" t="inlineStr">
-        <is>
-          <t>小阳线</t>
-        </is>
-      </c>
-      <c r="AI3" s="9" t="n">
-        <v>0</v>
-      </c>
       <c r="AJ3" s="11" t="n">
-        <v>3.22</v>
+        <v>2.96</v>
       </c>
       <c r="AK3" s="11" t="n">
-        <v>23.72</v>
-      </c>
-      <c r="AL3" s="15" t="inlineStr">
-        <is>
-          <t>趋势形成中</t>
+        <v>18.96</v>
+      </c>
+      <c r="AL3" s="8" t="inlineStr">
+        <is>
+          <t>无趋势</t>
         </is>
       </c>
       <c r="AM3" s="9" t="inlineStr">
@@ -2454,14 +2566,14 @@
         </is>
       </c>
       <c r="AN3" s="11" t="n">
-        <v>8.720000000000001</v>
+        <v>19.5</v>
       </c>
       <c r="AO3" s="11" t="n">
-        <v>4.28</v>
-      </c>
-      <c r="AP3" s="15" t="inlineStr">
-        <is>
-          <t>低波动平稳期</t>
+        <v>7.32</v>
+      </c>
+      <c r="AP3" s="14" t="inlineStr">
+        <is>
+          <t>健康趋势行情</t>
         </is>
       </c>
       <c r="AQ3" s="9" t="inlineStr">
@@ -2470,30 +2582,30 @@
         </is>
       </c>
       <c r="AR3" s="11" t="n">
-        <v>0.917</v>
+        <v>1.049</v>
       </c>
       <c r="AS3" s="11" t="n">
-        <v>1.022</v>
+        <v>1.091</v>
       </c>
       <c r="AT3" s="11" t="n">
-        <v>1.046</v>
+        <v>0.991</v>
       </c>
       <c r="AU3" s="11" t="n">
-        <v>0.892</v>
+        <v>1.079</v>
       </c>
       <c r="AV3" s="11" t="n">
-        <v>0.917</v>
-      </c>
-      <c r="AW3" s="15" t="inlineStr">
-        <is>
-          <t>强弱不明，震荡</t>
+        <v>1.049</v>
+      </c>
+      <c r="AW3" s="14" t="inlineStr">
+        <is>
+          <t>总体偏强</t>
         </is>
       </c>
       <c r="AX3" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AY3" s="11" t="n">
-        <v>2.29</v>
+        <v>2.47</v>
       </c>
       <c r="AZ3" s="9" t="n">
         <v>0</v>
@@ -2509,21 +2621,21 @@
         </is>
       </c>
       <c r="BC3" s="11" t="n">
-        <v>36.22</v>
-      </c>
-      <c r="BD3" s="15" t="inlineStr">
-        <is>
-          <t>偏弱区</t>
+        <v>25.61</v>
+      </c>
+      <c r="BD3" s="8" t="inlineStr">
+        <is>
+          <t>超卖区</t>
         </is>
       </c>
       <c r="BE3" s="11" t="n">
-        <v>25.21</v>
+        <v>40.85</v>
       </c>
       <c r="BF3" s="11" t="n">
-        <v>21.54</v>
+        <v>26.2</v>
       </c>
       <c r="BG3" s="11" t="n">
-        <v>32.54</v>
+        <v>70.16</v>
       </c>
       <c r="BH3" s="14" t="inlineStr">
         <is>
@@ -2531,10 +2643,10 @@
         </is>
       </c>
       <c r="BI3" s="11" t="n">
-        <v>-33.28</v>
+        <v>-19.12</v>
       </c>
       <c r="BJ3" s="11" t="n">
-        <v>45.91</v>
+        <v>46.43</v>
       </c>
       <c r="BK3" s="9" t="inlineStr">
         <is>
@@ -2543,40 +2655,44 @@
       </c>
       <c r="BL3" s="9" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="BM3" s="9" t="inlineStr">
         <is>
-          <t>MACD金叉</t>
-        </is>
-      </c>
-      <c r="BN3" s="9" t="inlineStr"/>
+          <t>超跌蓄势</t>
+        </is>
+      </c>
+      <c r="BN3" s="9" t="inlineStr">
+        <is>
+          <t>超跌蓄势</t>
+        </is>
+      </c>
       <c r="BO3" s="7" t="inlineStr">
         <is>
-          <t>深回撤|弱市</t>
+          <t>弱市</t>
         </is>
       </c>
       <c r="BP3" s="11" t="n">
-        <v>9.013999999999999</v>
+        <v>20.566</v>
       </c>
       <c r="BQ3" s="11" t="n">
-        <v>9.050000000000001</v>
+        <v>20.499</v>
       </c>
       <c r="BR3" s="11" t="n">
-        <v>9.044</v>
+        <v>20.755</v>
       </c>
       <c r="BS3" s="11" t="n">
-        <v>9.624000000000001</v>
+        <v>22.023</v>
       </c>
       <c r="BT3" s="11" t="n">
-        <v>11.024</v>
+        <v>22.67</v>
       </c>
       <c r="BU3" s="11" t="n">
         <v>0</v>
       </c>
       <c r="BV3" s="11" t="n">
-        <v>1.07</v>
+        <v>2.3</v>
       </c>
       <c r="BW3" s="14" t="inlineStr">
         <is>
@@ -2584,7 +2700,7 @@
         </is>
       </c>
       <c r="BX3" s="11" t="n">
-        <v>0.73</v>
+        <v>1.37</v>
       </c>
       <c r="BY3" s="14" t="inlineStr">
         <is>
@@ -2592,7 +2708,7 @@
         </is>
       </c>
       <c r="BZ3" s="11" t="n">
-        <v>-5.34</v>
+        <v>-4.46</v>
       </c>
       <c r="CA3" s="14" t="inlineStr">
         <is>
@@ -2600,21 +2716,21 @@
         </is>
       </c>
       <c r="CB3" s="11" t="n">
-        <v>-17.36</v>
-      </c>
-      <c r="CC3" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
+        <v>-7.19</v>
+      </c>
+      <c r="CC3" s="14" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="CD3" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CE3" s="9" t="n">
         <v>0</v>
       </c>
       <c r="CF3" s="9" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="CG3" s="9" t="n">
         <v>5</v>
@@ -2623,16 +2739,16 @@
         <v>5</v>
       </c>
       <c r="CI3" s="9" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="CJ3" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CK3" s="9" t="n">
         <v>0</v>
       </c>
       <c r="CL3" s="9" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="CM3" s="6" t="inlineStr">
         <is>
@@ -2645,10 +2761,10 @@
         </is>
       </c>
       <c r="CO3" s="11" t="n">
-        <v>80</v>
+        <v>85.7</v>
       </c>
       <c r="CP3" s="11" t="n">
-        <v>60</v>
+        <v>57.1</v>
       </c>
       <c r="CQ3" s="9" t="inlineStr">
         <is>
@@ -2659,16 +2775,16 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>SZ002028</t>
+          <t>SZ002271</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>思源电气</t>
+          <t>东方雨虹</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>112.59</v>
+        <v>10.71</v>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
@@ -2676,31 +2792,31 @@
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>125.1</v>
+        <v>10.64</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>125</v>
+        <v>10.65</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>125.09</v>
+        <v>10.8</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>112.59</v>
+        <v>10.58</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>116.76</v>
-      </c>
-      <c r="J4" s="13" t="n">
-        <v>-10</v>
+        <v>10.7</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>0.66</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>9.99</v>
+        <v>2.07</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>2.24</v>
+        <v>0.78</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0.23</v>
+        <v>0.03</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -2708,252 +2824,248 @@
         </is>
       </c>
       <c r="O4" s="4" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U4" s="13" t="n">
+        <v>-1.02</v>
+      </c>
+      <c r="V4" s="4" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="W4" s="4" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="Y4" s="4" t="n">
+        <v>10.71</v>
+      </c>
+      <c r="Z4" s="4" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="AA4" s="5" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="AB4" s="4" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="AC4" s="4" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="AD4" s="4" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="AE4" s="4" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="AF4" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AG4" s="2" t="inlineStr">
+        <is>
+          <t>站上 MA20</t>
+        </is>
+      </c>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>小阳线</t>
+        </is>
+      </c>
+      <c r="AI4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ4" s="4" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="AK4" s="4" t="n">
+        <v>9.880000000000001</v>
+      </c>
+      <c r="AL4" s="8" t="inlineStr">
+        <is>
+          <t>无趋势</t>
+        </is>
+      </c>
+      <c r="AM4" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AN4" s="4" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="AO4" s="4" t="n">
         <v>3.36</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" s="13" t="n">
-        <v>-4.61</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>6.75</v>
-      </c>
-      <c r="W4" s="4" t="n">
-        <v>118.57</v>
-      </c>
-      <c r="X4" s="4" t="n">
-        <v>125</v>
-      </c>
-      <c r="Y4" s="4" t="n">
-        <v>112.59</v>
-      </c>
-      <c r="Z4" s="4" t="n">
-        <v>124.13</v>
-      </c>
-      <c r="AA4" s="13" t="n">
-        <v>-9.300000000000001</v>
-      </c>
-      <c r="AB4" s="4" t="n">
-        <v>112.02</v>
-      </c>
-      <c r="AC4" s="4" t="n">
-        <v>125.95</v>
-      </c>
-      <c r="AD4" s="4" t="n">
-        <v>112.02</v>
-      </c>
-      <c r="AE4" s="4" t="n">
-        <v>125.95</v>
-      </c>
-      <c r="AF4" s="2" t="inlineStr">
-        <is>
-          <t>是（最近金叉）</t>
-        </is>
-      </c>
-      <c r="AG4" s="2" t="inlineStr">
-        <is>
-          <t>无明显形态</t>
-        </is>
-      </c>
-      <c r="AH4" s="2" t="inlineStr">
-        <is>
-          <t>光头大阴</t>
-        </is>
-      </c>
-      <c r="AI4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ4" s="4" t="n">
-        <v>3.91</v>
-      </c>
-      <c r="AK4" s="4" t="n">
-        <v>32.57</v>
-      </c>
-      <c r="AL4" s="14" t="inlineStr">
-        <is>
-          <t>强趋势</t>
-        </is>
-      </c>
-      <c r="AM4" s="2" t="inlineStr">
+      <c r="AP4" s="15" t="inlineStr">
+        <is>
+          <t>低波动平稳期</t>
+        </is>
+      </c>
+      <c r="AQ4" s="2" t="inlineStr">
+        <is>
+          <t>下降</t>
+        </is>
+      </c>
+      <c r="AR4" s="4" t="n">
+        <v>1.066</v>
+      </c>
+      <c r="AS4" s="4" t="n">
+        <v>1.008</v>
+      </c>
+      <c r="AT4" s="4" t="n">
+        <v>1.052</v>
+      </c>
+      <c r="AU4" s="4" t="n">
+        <v>1.121</v>
+      </c>
+      <c r="AV4" s="4" t="n">
+        <v>1.066</v>
+      </c>
+      <c r="AW4" s="14" t="inlineStr">
+        <is>
+          <t>总体偏强</t>
+        </is>
+      </c>
+      <c r="AX4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA4" s="2" t="inlineStr">
+        <is>
+          <t>主板</t>
+        </is>
+      </c>
+      <c r="BB4" s="2" t="inlineStr">
+        <is>
+          <t>沪深300</t>
+        </is>
+      </c>
+      <c r="BC4" s="4" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="BD4" s="14" t="inlineStr">
+        <is>
+          <t>偏强区</t>
+        </is>
+      </c>
+      <c r="BE4" s="4" t="n">
+        <v>58.09</v>
+      </c>
+      <c r="BF4" s="4" t="n">
+        <v>62.88</v>
+      </c>
+      <c r="BG4" s="4" t="n">
+        <v>48.53</v>
+      </c>
+      <c r="BH4" s="15" t="inlineStr">
+        <is>
+          <t>偏空</t>
+        </is>
+      </c>
+      <c r="BI4" s="4" t="n">
+        <v>-15.89</v>
+      </c>
+      <c r="BJ4" s="4" t="n">
+        <v>31.36</v>
+      </c>
+      <c r="BK4" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="AN4" s="4" t="n">
-        <v>112.02</v>
-      </c>
-      <c r="AO4" s="4" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="AP4" s="8" t="inlineStr">
-        <is>
-          <t>极低波动盘整</t>
-        </is>
-      </c>
-      <c r="AQ4" s="2" t="inlineStr">
-        <is>
-          <t>下降</t>
-        </is>
-      </c>
-      <c r="AR4" s="4" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="AS4" s="4" t="n">
-        <v>1.079</v>
-      </c>
-      <c r="AT4" s="4" t="n">
-        <v>1.078</v>
-      </c>
-      <c r="AU4" s="4" t="n">
-        <v>1.003</v>
-      </c>
-      <c r="AV4" s="4" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="AW4" s="14" t="inlineStr">
-        <is>
-          <t>总体偏强</t>
-        </is>
-      </c>
-      <c r="AX4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY4" s="4" t="n">
-        <v>1.79</v>
-      </c>
-      <c r="AZ4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA4" s="2" t="inlineStr">
-        <is>
-          <t>主板</t>
-        </is>
-      </c>
-      <c r="BB4" s="2" t="inlineStr">
-        <is>
-          <t>沪深300</t>
-        </is>
-      </c>
-      <c r="BC4" s="4" t="n">
-        <v>30.44</v>
-      </c>
-      <c r="BD4" s="15" t="inlineStr">
-        <is>
-          <t>偏弱区</t>
-        </is>
-      </c>
-      <c r="BE4" s="4" t="n">
-        <v>37.25</v>
-      </c>
-      <c r="BF4" s="4" t="n">
-        <v>35.32</v>
-      </c>
-      <c r="BG4" s="4" t="n">
-        <v>41.1</v>
-      </c>
-      <c r="BH4" s="14" t="inlineStr">
-        <is>
-          <t>偏多</t>
-        </is>
-      </c>
-      <c r="BI4" s="4" t="n">
-        <v>-38.53</v>
-      </c>
-      <c r="BJ4" s="4" t="n">
-        <v>56.19</v>
-      </c>
-      <c r="BK4" s="2" t="inlineStr">
+      <c r="BL4" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="BL4" s="2" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="BM4" s="2" t="inlineStr">
-        <is>
-          <t>MACD金叉</t>
-        </is>
-      </c>
+      <c r="BM4" s="2" t="inlineStr"/>
       <c r="BN4" s="2" t="inlineStr"/>
       <c r="BO4" s="7" t="inlineStr">
         <is>
-          <t>深回撤|弱市</t>
+          <t>弱市</t>
         </is>
       </c>
       <c r="BP4" s="4" t="n">
-        <v>117.76</v>
+        <v>10.696</v>
       </c>
       <c r="BQ4" s="4" t="n">
-        <v>118.307</v>
+        <v>10.706</v>
       </c>
       <c r="BR4" s="4" t="n">
-        <v>118.581</v>
+        <v>10.734</v>
       </c>
       <c r="BS4" s="4" t="n">
-        <v>124.747</v>
+        <v>10.584</v>
       </c>
       <c r="BT4" s="4" t="n">
-        <v>146.681</v>
+        <v>11.05</v>
       </c>
       <c r="BU4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="BV4" s="4" t="n">
-        <v>-4.39</v>
-      </c>
-      <c r="BW4" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
+        <v>0.13</v>
+      </c>
+      <c r="BW4" s="14" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="BX4" s="4" t="n">
-        <v>-5.05</v>
-      </c>
-      <c r="BY4" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
+        <v>-0.22</v>
+      </c>
+      <c r="BY4" s="14" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="BZ4" s="4" t="n">
-        <v>-9.74</v>
-      </c>
-      <c r="CA4" s="8" t="inlineStr">
-        <is>
-          <t>超卖偏弱</t>
+        <v>1.19</v>
+      </c>
+      <c r="CA4" s="14" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="CB4" s="4" t="n">
-        <v>-23.24</v>
-      </c>
-      <c r="CC4" s="8" t="inlineStr">
-        <is>
-          <t>极度超卖</t>
+        <v>-3.07</v>
+      </c>
+      <c r="CC4" s="14" t="inlineStr">
+        <is>
+          <t>中性区间</t>
         </is>
       </c>
       <c r="CD4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="CE4" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CF4" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="CG4" s="2" t="n">
         <v>5</v>
@@ -2962,16 +3074,16 @@
         <v>5</v>
       </c>
       <c r="CI4" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="CJ4" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CK4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="CL4" s="2" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="CM4" s="6" t="inlineStr">
         <is>
@@ -2984,10 +3096,10 @@
         </is>
       </c>
       <c r="CO4" s="4" t="n">
-        <v>50</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="CP4" s="4" t="n">
-        <v>40</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="CQ4" s="2" t="inlineStr">
         <is>
@@ -2998,16 +3110,16 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>SZ002240</t>
+          <t>SZ002460</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>盛新锂能</t>
+          <t>赣锋锂业</t>
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>21.5</v>
+        <v>37.8</v>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
@@ -3015,31 +3127,31 @@
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>21.34</v>
+        <v>38.23</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>21.1</v>
+        <v>37.85</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>21.82</v>
+        <v>38.71</v>
       </c>
       <c r="H5" s="11" t="n">
-        <v>20.95</v>
+        <v>37.32</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>21.42</v>
+        <v>37.94</v>
       </c>
       <c r="J5" s="12" t="n">
-        <v>0.75</v>
+        <v>-1.12</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>4.08</v>
+        <v>3.64</v>
       </c>
       <c r="L5" s="11" t="n">
-        <v>0.79</v>
+        <v>1.07</v>
       </c>
       <c r="M5" s="11" t="n">
-        <v>0.04</v>
+        <v>17.87</v>
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
@@ -3047,10 +3159,10 @@
         </is>
       </c>
       <c r="O5" s="11" t="n">
-        <v>1.89</v>
+        <v>3.9</v>
       </c>
       <c r="P5" s="11" t="n">
-        <v>0.17</v>
+        <v>47.23</v>
       </c>
       <c r="Q5" s="11" t="n">
         <v>0</v>
@@ -3062,40 +3174,40 @@
         <v>0</v>
       </c>
       <c r="T5" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U5" s="12" t="n">
-        <v>0.23</v>
+        <v>-3.79</v>
       </c>
       <c r="V5" s="11" t="n">
-        <v>3.98</v>
+        <v>4.45</v>
       </c>
       <c r="W5" s="11" t="n">
-        <v>21.43</v>
+        <v>38.44</v>
       </c>
       <c r="X5" s="11" t="n">
-        <v>21.1</v>
+        <v>37.85</v>
       </c>
       <c r="Y5" s="11" t="n">
-        <v>21.5</v>
+        <v>37.8</v>
       </c>
       <c r="Z5" s="11" t="n">
-        <v>24.78</v>
-      </c>
-      <c r="AA5" s="16" t="n">
-        <v>-13.24</v>
+        <v>42.77</v>
+      </c>
+      <c r="AA5" s="12" t="n">
+        <v>-11.62</v>
       </c>
       <c r="AB5" s="11" t="n">
-        <v>20.9</v>
+        <v>37.32</v>
       </c>
       <c r="AC5" s="11" t="n">
-        <v>25.95</v>
+        <v>46.1</v>
       </c>
       <c r="AD5" s="11" t="n">
-        <v>20.9</v>
+        <v>37.32</v>
       </c>
       <c r="AE5" s="11" t="n">
-        <v>23.44</v>
+        <v>42.39</v>
       </c>
       <c r="AF5" s="9" t="inlineStr">
         <is>
@@ -3109,21 +3221,21 @@
       </c>
       <c r="AH5" s="9" t="inlineStr">
         <is>
-          <t>看涨吞没</t>
+          <t>十字星</t>
         </is>
       </c>
       <c r="AI5" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AJ5" s="11" t="n">
-        <v>3.32</v>
+        <v>3.31</v>
       </c>
       <c r="AK5" s="11" t="n">
-        <v>43.64</v>
+        <v>37.24</v>
       </c>
       <c r="AL5" s="14" t="inlineStr">
         <is>
-          <t>极强趋势</t>
+          <t>强趋势</t>
         </is>
       </c>
       <c r="AM5" s="9" t="inlineStr">
@@ -3132,10 +3244,10 @@
         </is>
       </c>
       <c r="AN5" s="11" t="n">
-        <v>20.9</v>
+        <v>37.32</v>
       </c>
       <c r="AO5" s="11" t="n">
-        <v>2.79</v>
+        <v>1.27</v>
       </c>
       <c r="AP5" s="8" t="inlineStr">
         <is>
@@ -3148,19 +3260,19 @@
         </is>
       </c>
       <c r="AR5" s="11" t="n">
-        <v>0.904</v>
+        <v>0.905</v>
       </c>
       <c r="AS5" s="11" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="AT5" s="11" t="n">
-        <v>0.887</v>
+        <v>0.913</v>
       </c>
       <c r="AU5" s="11" t="n">
-        <v>0.842</v>
+        <v>0.889</v>
       </c>
       <c r="AV5" s="11" t="n">
-        <v>0.904</v>
+        <v>0.905</v>
       </c>
       <c r="AW5" s="8" t="inlineStr">
         <is>
@@ -3171,7 +3283,7 @@
         <v>0</v>
       </c>
       <c r="AY5" s="11" t="n">
-        <v>2.43</v>
+        <v>2.9</v>
       </c>
       <c r="AZ5" s="9" t="n">
         <v>0</v>
@@ -3187,32 +3299,32 @@
         </is>
       </c>
       <c r="BC5" s="11" t="n">
-        <v>13.59</v>
+        <v>22.7</v>
       </c>
       <c r="BD5" s="8" t="inlineStr">
         <is>
+          <t>超卖区</t>
+        </is>
+      </c>
+      <c r="BE5" s="11" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="BF5" s="11" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="BG5" s="11" t="n">
+        <v>-3.14</v>
+      </c>
+      <c r="BH5" s="8" t="inlineStr">
+        <is>
           <t>极度超卖</t>
         </is>
       </c>
-      <c r="BE5" s="11" t="n">
-        <v>9.470000000000001</v>
-      </c>
-      <c r="BF5" s="11" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="BG5" s="11" t="n">
-        <v>6.52</v>
-      </c>
-      <c r="BH5" s="8" t="inlineStr">
-        <is>
-          <t>低位钝化</t>
-        </is>
-      </c>
       <c r="BI5" s="11" t="n">
-        <v>-37.03</v>
+        <v>-32.05</v>
       </c>
       <c r="BJ5" s="11" t="n">
-        <v>38.39</v>
+        <v>35.77</v>
       </c>
       <c r="BK5" s="9" t="inlineStr">
         <is>
@@ -3232,41 +3344,41 @@
         </is>
       </c>
       <c r="BP5" s="11" t="n">
-        <v>21.752</v>
+        <v>39.266</v>
       </c>
       <c r="BQ5" s="11" t="n">
-        <v>22.231</v>
+        <v>40.277</v>
       </c>
       <c r="BR5" s="11" t="n">
-        <v>23.112</v>
+        <v>41.505</v>
       </c>
       <c r="BS5" s="11" t="n">
-        <v>24.779</v>
+        <v>43.294</v>
       </c>
       <c r="BT5" s="11" t="n">
-        <v>28.626</v>
+        <v>48.663</v>
       </c>
       <c r="BU5" s="11" t="n">
         <v>0</v>
       </c>
       <c r="BV5" s="11" t="n">
-        <v>-1.16</v>
-      </c>
-      <c r="BW5" s="14" t="inlineStr">
-        <is>
-          <t>中性区间</t>
+        <v>-3.73</v>
+      </c>
+      <c r="BW5" s="8" t="inlineStr">
+        <is>
+          <t>超卖偏弱</t>
         </is>
       </c>
       <c r="BX5" s="11" t="n">
-        <v>-6.97</v>
+        <v>-8.93</v>
       </c>
       <c r="BY5" s="8" t="inlineStr">
         <is>
-          <t>超卖偏弱</t>
+          <t>极度超卖</t>
         </is>
       </c>
       <c r="BZ5" s="11" t="n">
-        <v>-13.23</v>
+        <v>-12.69</v>
       </c>
       <c r="CA5" s="8" t="inlineStr">
         <is>
@@ -3274,7 +3386,7 @@
         </is>
       </c>
       <c r="CB5" s="11" t="n">
-        <v>-24.89</v>
+        <v>-22.32</v>
       </c>
       <c r="CC5" s="8" t="inlineStr">
         <is>
@@ -3322,7 +3434,7 @@
         <v>50</v>
       </c>
       <c r="CP5" s="11" t="n">
-        <v>20</v>
+        <v>28.6</v>
       </c>
       <c r="CQ5" s="9" t="inlineStr">
         <is>
@@ -3333,16 +3445,16 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SZ002223</t>
+          <t>SZ002466</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>鱼跃医疗</t>
+          <t>天齐锂业</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>25.66</v>
+        <v>36.5</v>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
@@ -3350,31 +3462,31 @@
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>25.9</v>
+        <v>36.43</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>25.93</v>
+        <v>36.11</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>26</v>
+        <v>36.9</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>25.43</v>
+        <v>35.91</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>25.7</v>
-      </c>
-      <c r="J6" s="13" t="n">
-        <v>-0.93</v>
+        <v>36.44</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>0.19</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>2.2</v>
+        <v>2.72</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.72</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>0.02</v>
+        <v>6.73</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -3382,10 +3494,10 @@
         </is>
       </c>
       <c r="O6" s="4" t="n">
-        <v>0.98</v>
+        <v>1.25</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>0.09</v>
+        <v>18.49</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>0</v>
@@ -3397,40 +3509,40 @@
         <v>0</v>
       </c>
       <c r="T6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U6" s="5" t="n">
-        <v>1.7</v>
+        <v>0.16</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>3.4</v>
+        <v>2.97</v>
       </c>
       <c r="W6" s="4" t="n">
-        <v>25.6</v>
+        <v>36.46</v>
       </c>
       <c r="X6" s="4" t="n">
-        <v>25.93</v>
+        <v>36.11</v>
       </c>
       <c r="Y6" s="4" t="n">
-        <v>25.66</v>
+        <v>36.5</v>
       </c>
       <c r="Z6" s="4" t="n">
-        <v>26.05</v>
+        <v>40.28</v>
       </c>
       <c r="AA6" s="13" t="n">
-        <v>-1.5</v>
+        <v>-9.380000000000001</v>
       </c>
       <c r="AB6" s="4" t="n">
-        <v>24.94</v>
+        <v>35.9</v>
       </c>
       <c r="AC6" s="4" t="n">
-        <v>26.68</v>
+        <v>41.81</v>
       </c>
       <c r="AD6" s="4" t="n">
-        <v>24.94</v>
+        <v>35.9</v>
       </c>
       <c r="AE6" s="4" t="n">
-        <v>26.44</v>
+        <v>38.9</v>
       </c>
       <c r="AF6" s="2" t="inlineStr">
         <is>
@@ -3444,21 +3556,21 @@
       </c>
       <c r="AH6" s="2" t="inlineStr">
         <is>
-          <t>小阴线</t>
+          <t>看涨吞没</t>
         </is>
       </c>
       <c r="AI6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>3.75</v>
+        <v>4.18</v>
       </c>
       <c r="AK6" s="4" t="n">
-        <v>14.72</v>
-      </c>
-      <c r="AL6" s="8" t="inlineStr">
-        <is>
-          <t>无趋势</t>
+        <v>37.33</v>
+      </c>
+      <c r="AL6" s="14" t="inlineStr">
+        <is>
+          <t>强趋势</t>
         </is>
       </c>
       <c r="AM6" s="2" t="inlineStr">
@@ -3467,10 +3579,10 @@
         </is>
       </c>
       <c r="AN6" s="4" t="n">
-        <v>24.94</v>
+        <v>35.9</v>
       </c>
       <c r="AO6" s="4" t="n">
-        <v>2.81</v>
+        <v>1.64</v>
       </c>
       <c r="AP6" s="8" t="inlineStr">
         <is>
@@ -3483,30 +3595,30 @@
         </is>
       </c>
       <c r="AR6" s="4" t="n">
-        <v>1.042</v>
+        <v>0.954</v>
       </c>
       <c r="AS6" s="4" t="n">
-        <v>1.01</v>
+        <v>0.983</v>
       </c>
       <c r="AT6" s="4" t="n">
-        <v>1.05</v>
+        <v>0.952</v>
       </c>
       <c r="AU6" s="4" t="n">
-        <v>1.09</v>
+        <v>0.929</v>
       </c>
       <c r="AV6" s="4" t="n">
-        <v>1.042</v>
-      </c>
-      <c r="AW6" s="14" t="inlineStr">
-        <is>
-          <t>总体偏强</t>
+        <v>0.954</v>
+      </c>
+      <c r="AW6" s="8" t="inlineStr">
+        <is>
+          <t>总体偏弱</t>
         </is>
       </c>
       <c r="AX6" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AY6" s="4" t="n">
-        <v>0.99</v>
+        <v>1.8</v>
       </c>
       <c r="AZ6" s="2" t="n">
         <v>0</v>
@@ -3522,32 +3634,32 @@
         </is>
       </c>
       <c r="BC6" s="4" t="n">
-        <v>41.43</v>
-      </c>
-      <c r="BD6" s="15" t="inlineStr">
-        <is>
-          <t>偏弱区</t>
+        <v>20.66</v>
+      </c>
+      <c r="BD6" s="8" t="inlineStr">
+        <is>
+          <t>超卖区</t>
         </is>
       </c>
       <c r="BE6" s="4" t="n">
-        <v>40.81</v>
+        <v>10.58</v>
       </c>
       <c r="BF6" s="4" t="n">
-        <v>42.53</v>
+        <v>13.51</v>
       </c>
       <c r="BG6" s="4" t="n">
-        <v>37.37</v>
-      </c>
-      <c r="BH6" s="15" t="inlineStr">
-        <is>
-          <t>偏空</t>
+        <v>4.73</v>
+      </c>
+      <c r="BH6" s="8" t="inlineStr">
+        <is>
+          <t>低位钝化</t>
         </is>
       </c>
       <c r="BI6" s="4" t="n">
-        <v>-9.69</v>
+        <v>-27.29</v>
       </c>
       <c r="BJ6" s="4" t="n">
-        <v>23.57</v>
+        <v>31.33</v>
       </c>
       <c r="BK6" s="2" t="inlineStr">
         <is>
@@ -3563,29 +3675,29 @@
       <c r="BN6" s="2" t="inlineStr"/>
       <c r="BO6" s="7" t="inlineStr">
         <is>
-          <t>弱市</t>
+          <t>深回撤|弱市</t>
         </is>
       </c>
       <c r="BP6" s="4" t="n">
-        <v>25.656</v>
+        <v>36.774</v>
       </c>
       <c r="BQ6" s="4" t="n">
-        <v>25.887</v>
+        <v>37.371</v>
       </c>
       <c r="BR6" s="4" t="n">
-        <v>25.955</v>
+        <v>38.391</v>
       </c>
       <c r="BS6" s="4" t="n">
-        <v>26.098</v>
+        <v>40.176</v>
       </c>
       <c r="BT6" s="4" t="n">
-        <v>26.227</v>
+        <v>44.503</v>
       </c>
       <c r="BU6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="BV6" s="4" t="n">
-        <v>0.02</v>
+        <v>-0.75</v>
       </c>
       <c r="BW6" s="14" t="inlineStr">
         <is>
@@ -3593,7 +3705,7 @@
         </is>
       </c>
       <c r="BX6" s="4" t="n">
-        <v>-1.14</v>
+        <v>-4.93</v>
       </c>
       <c r="BY6" s="14" t="inlineStr">
         <is>
@@ -3601,19 +3713,19 @@
         </is>
       </c>
       <c r="BZ6" s="4" t="n">
-        <v>-1.68</v>
-      </c>
-      <c r="CA6" s="14" t="inlineStr">
-        <is>
-          <t>中性区间</t>
+        <v>-9.15</v>
+      </c>
+      <c r="CA6" s="8" t="inlineStr">
+        <is>
+          <t>超卖偏弱</t>
         </is>
       </c>
       <c r="CB6" s="4" t="n">
-        <v>-2.16</v>
-      </c>
-      <c r="CC6" s="14" t="inlineStr">
-        <is>
-          <t>中性区间</t>
+        <v>-17.98</v>
+      </c>
+      <c r="CC6" s="8" t="inlineStr">
+        <is>
+          <t>超卖偏弱</t>
         </is>
       </c>
       <c r="CD6" s="2" t="n">
@@ -3623,7 +3735,7 @@
         <v>0</v>
       </c>
       <c r="CF6" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="CG6" s="2" t="n">
         <v>5</v>
@@ -3635,38 +3747,708 @@
         <v>0</v>
       </c>
       <c r="CJ6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL6" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="CM6" s="6" t="inlineStr">
+        <is>
+          <t>D 级 (风险)</t>
+        </is>
+      </c>
+      <c r="CN6" s="2" t="inlineStr">
+        <is>
+          <t>排除/止损 | 弱市慎加仓</t>
+        </is>
+      </c>
+      <c r="CO6" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="CP6" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="CQ6" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>SZ002245</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>蔚蓝锂芯</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>12.87</v>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>弱势</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>14.23</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>14.24</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>12.87</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>13.33</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>-10</v>
+      </c>
+      <c r="K7" s="11" t="n">
+        <v>9.58</v>
+      </c>
+      <c r="L7" s="11" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="M7" s="11" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="N7" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="O7" s="11" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="P7" s="11" t="n">
+        <v>140.14</v>
+      </c>
+      <c r="Q7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="12" t="n">
+        <v>-9.81</v>
+      </c>
+      <c r="V7" s="11" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="W7" s="11" t="n">
+        <v>13.81</v>
+      </c>
+      <c r="X7" s="11" t="n">
+        <v>14.23</v>
+      </c>
+      <c r="Y7" s="11" t="n">
+        <v>12.87</v>
+      </c>
+      <c r="Z7" s="11" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="AA7" s="12" t="n">
+        <v>-19.06</v>
+      </c>
+      <c r="AB7" s="11" t="n">
+        <v>12.87</v>
+      </c>
+      <c r="AC7" s="11" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="AD7" s="11" t="n">
+        <v>12.87</v>
+      </c>
+      <c r="AE7" s="11" t="n">
+        <v>15.74</v>
+      </c>
+      <c r="AF7" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AG7" s="9" t="inlineStr">
+        <is>
+          <t>无明显形态</t>
+        </is>
+      </c>
+      <c r="AH7" s="9" t="inlineStr">
+        <is>
+          <t>光头大阴</t>
+        </is>
+      </c>
+      <c r="AI7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" s="11" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="AK7" s="11" t="n">
+        <v>17.69</v>
+      </c>
+      <c r="AL7" s="8" t="inlineStr">
+        <is>
+          <t>无趋势</t>
+        </is>
+      </c>
+      <c r="AM7" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AN7" s="11" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="AO7" s="11" t="n">
+        <v>19.97</v>
+      </c>
+      <c r="AP7" s="7" t="inlineStr">
+        <is>
+          <t>剧烈波动/深回撤中</t>
+        </is>
+      </c>
+      <c r="AQ7" s="9" t="inlineStr">
+        <is>
+          <t>下降</t>
+        </is>
+      </c>
+      <c r="AR7" s="11" t="n">
+        <v>0.853</v>
+      </c>
+      <c r="AS7" s="11" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="AT7" s="11" t="n">
+        <v>0.836</v>
+      </c>
+      <c r="AU7" s="11" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="AV7" s="11" t="n">
+        <v>0.853</v>
+      </c>
+      <c r="AW7" s="8" t="inlineStr">
+        <is>
+          <t>总体偏弱</t>
+        </is>
+      </c>
+      <c r="AX7" s="9" t="n">
+        <v>-5</v>
+      </c>
+      <c r="AY7" s="11" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="AZ7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA7" s="9" t="inlineStr">
+        <is>
+          <t>主板</t>
+        </is>
+      </c>
+      <c r="BB7" s="9" t="inlineStr">
+        <is>
+          <t>沪深300</t>
+        </is>
+      </c>
+      <c r="BC7" s="11" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="BD7" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
+        </is>
+      </c>
+      <c r="BE7" s="11" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="BF7" s="11" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="BG7" s="11" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="BH7" s="8" t="inlineStr">
+        <is>
+          <t>低位钝化</t>
+        </is>
+      </c>
+      <c r="BI7" s="11" t="n">
+        <v>-33.83</v>
+      </c>
+      <c r="BJ7" s="11" t="n">
+        <v>41.74</v>
+      </c>
+      <c r="BK7" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="BL7" s="9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="BM7" s="9" t="inlineStr"/>
+      <c r="BN7" s="9" t="inlineStr"/>
+      <c r="BO7" s="7" t="inlineStr">
+        <is>
+          <t>深回撤|止损过宽|弱市</t>
+        </is>
+      </c>
+      <c r="BP7" s="11" t="n">
+        <v>14.162</v>
+      </c>
+      <c r="BQ7" s="11" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="BR7" s="11" t="n">
+        <v>15.08</v>
+      </c>
+      <c r="BS7" s="11" t="n">
+        <v>16.189</v>
+      </c>
+      <c r="BT7" s="11" t="n">
+        <v>17.032</v>
+      </c>
+      <c r="BU7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV7" s="11" t="n">
+        <v>-9.119999999999999</v>
+      </c>
+      <c r="BW7" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
+        </is>
+      </c>
+      <c r="BX7" s="11" t="n">
+        <v>-14.66</v>
+      </c>
+      <c r="BY7" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
+        </is>
+      </c>
+      <c r="BZ7" s="11" t="n">
+        <v>-20.5</v>
+      </c>
+      <c r="CA7" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
+        </is>
+      </c>
+      <c r="CB7" s="11" t="n">
+        <v>-24.43</v>
+      </c>
+      <c r="CC7" s="8" t="inlineStr">
+        <is>
+          <t>极度超卖</t>
+        </is>
+      </c>
+      <c r="CD7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF7" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="CK6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="CL6" s="2" t="n">
+      <c r="CG7" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="CH7" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="CI7" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="CJ7" s="9" t="n">
+        <v>-5</v>
+      </c>
+      <c r="CK7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL7" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="CM6" s="6" t="inlineStr">
+      <c r="CM7" s="6" t="inlineStr">
         <is>
           <t>D 级 (风险)</t>
         </is>
       </c>
-      <c r="CN6" s="2" t="inlineStr">
+      <c r="CN7" s="9" t="inlineStr">
         <is>
           <t>排除/止损 | 弱市慎加仓</t>
         </is>
       </c>
-      <c r="CO6" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="CP6" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="CQ6" s="2" t="inlineStr">
+      <c r="CO7" s="11" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="CP7" s="11" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="CQ7" s="9" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SZ002223</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>鱼跃医疗</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>25.66</v>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>弱势</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>25.93</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>25.43</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="J8" s="13" t="n">
+        <v>-0.93</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="5" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="V8" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="X8" s="4" t="n">
+        <v>25.93</v>
+      </c>
+      <c r="Y8" s="4" t="n">
+        <v>25.66</v>
+      </c>
+      <c r="Z8" s="4" t="n">
+        <v>26.05</v>
+      </c>
+      <c r="AA8" s="13" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="AB8" s="4" t="n">
+        <v>24.94</v>
+      </c>
+      <c r="AC8" s="4" t="n">
+        <v>26.68</v>
+      </c>
+      <c r="AD8" s="4" t="n">
+        <v>24.94</v>
+      </c>
+      <c r="AE8" s="4" t="n">
+        <v>26.44</v>
+      </c>
+      <c r="AF8" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AG8" s="2" t="inlineStr">
+        <is>
+          <t>无明显形态</t>
+        </is>
+      </c>
+      <c r="AH8" s="2" t="inlineStr">
+        <is>
+          <t>小阴线</t>
+        </is>
+      </c>
+      <c r="AI8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" s="4" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="AK8" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="AL8" s="8" t="inlineStr">
+        <is>
+          <t>无趋势</t>
+        </is>
+      </c>
+      <c r="AM8" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AN8" s="4" t="n">
+        <v>24.94</v>
+      </c>
+      <c r="AO8" s="4" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="AP8" s="8" t="inlineStr">
+        <is>
+          <t>极低波动盘整</t>
+        </is>
+      </c>
+      <c r="AQ8" s="2" t="inlineStr">
+        <is>
+          <t>下降</t>
+        </is>
+      </c>
+      <c r="AR8" s="4" t="n">
+        <v>1.081</v>
+      </c>
+      <c r="AS8" s="4" t="n">
+        <v>1.004</v>
+      </c>
+      <c r="AT8" s="4" t="n">
+        <v>1.025</v>
+      </c>
+      <c r="AU8" s="4" t="n">
+        <v>1.055</v>
+      </c>
+      <c r="AV8" s="4" t="n">
+        <v>1.081</v>
+      </c>
+      <c r="AW8" s="14" t="inlineStr">
+        <is>
+          <t>全面跑赢，强势确认</t>
+        </is>
+      </c>
+      <c r="AX8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY8" s="4" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AZ8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA8" s="2" t="inlineStr">
+        <is>
+          <t>主板</t>
+        </is>
+      </c>
+      <c r="BB8" s="2" t="inlineStr">
+        <is>
+          <t>沪深300</t>
+        </is>
+      </c>
+      <c r="BC8" s="4" t="n">
+        <v>41.43</v>
+      </c>
+      <c r="BD8" s="15" t="inlineStr">
+        <is>
+          <t>偏弱区</t>
+        </is>
+      </c>
+      <c r="BE8" s="4" t="n">
+        <v>40.81</v>
+      </c>
+      <c r="BF8" s="4" t="n">
+        <v>42.53</v>
+      </c>
+      <c r="BG8" s="4" t="n">
+        <v>37.37</v>
+      </c>
+      <c r="BH8" s="15" t="inlineStr">
+        <is>
+          <t>偏空</t>
+        </is>
+      </c>
+      <c r="BI8" s="4" t="n">
+        <v>-9.550000000000001</v>
+      </c>
+      <c r="BJ8" s="4" t="n">
+        <v>23.57</v>
+      </c>
+      <c r="BK8" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="BL8" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="BM8" s="2" t="inlineStr"/>
+      <c r="BN8" s="2" t="inlineStr"/>
+      <c r="BO8" s="7" t="inlineStr">
+        <is>
+          <t>弱市</t>
+        </is>
+      </c>
+      <c r="BP8" s="4" t="n">
+        <v>25.656</v>
+      </c>
+      <c r="BQ8" s="4" t="n">
+        <v>25.887</v>
+      </c>
+      <c r="BR8" s="4" t="n">
+        <v>25.955</v>
+      </c>
+      <c r="BS8" s="4" t="n">
+        <v>26.098</v>
+      </c>
+      <c r="BT8" s="4" t="n">
+        <v>26.22</v>
+      </c>
+      <c r="BU8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV8" s="4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BW8" s="14" t="inlineStr">
+        <is>
+          <t>中性区间</t>
+        </is>
+      </c>
+      <c r="BX8" s="4" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="BY8" s="14" t="inlineStr">
+        <is>
+          <t>中性区间</t>
+        </is>
+      </c>
+      <c r="BZ8" s="4" t="n">
+        <v>-1.68</v>
+      </c>
+      <c r="CA8" s="14" t="inlineStr">
+        <is>
+          <t>中性区间</t>
+        </is>
+      </c>
+      <c r="CB8" s="4" t="n">
+        <v>-2.14</v>
+      </c>
+      <c r="CC8" s="14" t="inlineStr">
+        <is>
+          <t>中性区间</t>
+        </is>
+      </c>
+      <c r="CD8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="CH8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="CI8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="CK8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL8" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="CM8" s="6" t="inlineStr">
+        <is>
+          <t>D 级 (风险)</t>
+        </is>
+      </c>
+      <c r="CN8" s="2" t="inlineStr">
+        <is>
+          <t>排除/止损 | 弱市慎加仓</t>
+        </is>
+      </c>
+      <c r="CO8" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="CP8" s="4" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="CQ8" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="CL2:CL6">
+  <conditionalFormatting sqref="CL2:CL8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="15"/>
@@ -3678,7 +4460,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="CO2:CO6">
+  <conditionalFormatting sqref="CO2:CO8">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -3690,7 +4472,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AR2:AR6">
+  <conditionalFormatting sqref="AR2:AR8">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -3702,7 +4484,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AS2:AS6">
+  <conditionalFormatting sqref="AS2:AS8">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -3714,7 +4496,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AT2:AT6">
+  <conditionalFormatting sqref="AT2:AT8">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -3726,7 +4508,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AU2:AU6">
+  <conditionalFormatting sqref="AU2:AU8">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -3738,7 +4520,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AV2:AV6">
+  <conditionalFormatting sqref="AV2:AV8">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -3750,7 +4532,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK2:AK6">
+  <conditionalFormatting sqref="AK2:AK8">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="num" val="15"/>
@@ -3862,7 +4644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3971,7 +4753,100 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SZ002241</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>歌尔股份</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>21.04</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>D 级 (风险)</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>弱势</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>超跌蓄势</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>超跌蓄势</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>弱市</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>25.61</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>70.16</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>-4.46</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>1.049</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>-19.12</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>46.43</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="D2">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="15"/>
+        <cfvo type="num" val="50"/>
+        <cfvo type="num" val="85"/>
+        <color rgb="00F1948A"/>
+        <color rgb="00F9E79F"/>
+        <color rgb="0082E0AA"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O2">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0.7"/>
+        <cfvo type="num" val="1"/>
+        <cfvo type="num" val="1.3"/>
+        <color rgb="00F1948A"/>
+        <color rgb="00F9E79F"/>
+        <color rgb="0082E0AA"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4543,7 +5418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4569,17 +5444,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>科创/创业板</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -4619,7 +5484,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -4633,7 +5498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4649,28 +5514,28 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SZ002245: SZ002245 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ000582: SZ000582 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>SZ002460: SZ002460 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ300831: SZ300831 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>SZ002466: SZ002466 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ002028: SZ002028 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>SZ000555: SZ000555 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ002240: SZ002240 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
@@ -4747,138 +5612,124 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>SZ002241: SZ002241 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ301358: SZ301358 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>SZ002271: SZ002271 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ300750: SZ300750 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>SZ301358: SZ301358 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ300442: SZ300442 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>SZ300750: SZ300750 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ002922: SZ002922 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>SZ300442: SZ300442 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ300919: SZ300919 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>SZ002922: SZ002922 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ300274: SZ300274 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>SZ300919: SZ300919 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ002709: SZ002709 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>SZ300274: SZ300274 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ001386: SZ001386 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>SZ002709: SZ002709 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ000657: SZ000657 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>SZ001386: SZ001386 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ300760: SZ300760 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SZ000657: SZ000657 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ300558: SZ300558 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>SZ300760: SZ300760 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ000788: SZ000788 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SZ300558: SZ300558 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ300404: SZ300404 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>SZ000788: SZ000788 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ002929: SZ002929 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SZ300404: SZ300404 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ300339: SZ300339 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>SZ002929: SZ002929 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ002202: SZ002202 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>SZ300339: SZ300339 数据获取失败（AkShare+Baostock均失败）</t>
+          <t>SZ000400: SZ000400 数据获取失败（AkShare+Baostock均失败）</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>SZ002202: SZ002202 数据获取失败（AkShare+Baostock均失败）</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>SZ000400: SZ000400 数据获取失败（AkShare+Baostock均失败）</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>SZ002866: SZ002866 数据获取失败（AkShare+Baostock均失败）</t>
         </is>

</xml_diff>

<commit_message>
auto stock scan 2026-10-28 14:46 UTC
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -2877,7 +2877,7 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="20.25" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
     <col width="15.875" customWidth="1" min="24" max="24"/>
@@ -3105,52 +3105,52 @@
         </is>
       </c>
       <c r="C3" s="12" t="n">
+        <v>11473.18</v>
+      </c>
+      <c r="D3" s="12" t="n">
         <v>11245.73</v>
       </c>
-      <c r="D3" s="12" t="n">
-        <v>11534.38</v>
-      </c>
       <c r="E3" s="12" t="n">
-        <v>11591.36</v>
+        <v>11359.08</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>11633.3</v>
+        <v>11529.59</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>11245.72</v>
-      </c>
-      <c r="H3" s="13" t="n">
-        <v>-2.5</v>
+        <v>11292.7</v>
+      </c>
+      <c r="H3" s="17" t="n">
+        <v>2.02</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>3.36</v>
+        <v>2.11</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>11503.122</v>
+        <v>11456.887</v>
       </c>
       <c r="K3" s="12" t="n">
-        <v>11686.416</v>
+        <v>11622.675</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>12720.471</v>
+        <v>12646.137</v>
       </c>
       <c r="M3" s="12" t="n">
-        <v>13337.735</v>
+        <v>13303.794</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>14336.337</v>
+        <v>14305.939</v>
       </c>
       <c r="O3" s="12" t="n">
         <v>11043.31</v>
       </c>
       <c r="P3" s="12" t="n">
-        <v>12383.62</v>
+        <v>11993.85</v>
       </c>
       <c r="Q3" s="12" t="n">
         <v>11043.31</v>
       </c>
       <c r="R3" s="12" t="n">
-        <v>11909.62</v>
+        <v>11707.15</v>
       </c>
       <c r="S3" s="10" t="inlineStr">
         <is>
@@ -3164,11 +3164,11 @@
       </c>
       <c r="U3" s="10" t="inlineStr">
         <is>
-          <t>光头大阴 | 黄昏之星 (见顶)</t>
+          <t>看涨孕线</t>
         </is>
       </c>
       <c r="V3" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W3" s="9" t="inlineStr">
         <is>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="X3" s="10" t="inlineStr">
         <is>
-          <t>跌破MA60 | 日内偏弱</t>
+          <t>跌破MA60 | 日内偏强</t>
         </is>
       </c>
     </row>
@@ -3193,40 +3193,40 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
+        <v>23094.83</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>23041.32</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>23211.81</v>
-      </c>
       <c r="E4" s="4" t="n">
-        <v>23260.14</v>
+        <v>23083.99</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>23313.92</v>
+        <v>23157.4</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>22983.99</v>
-      </c>
-      <c r="H4" s="16" t="n">
-        <v>-0.73</v>
+        <v>23023.04</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>0.23</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1.42</v>
+        <v>0.58</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>23186.61</v>
+        <v>23075.202</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>23670.973</v>
+        <v>23545.934</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>24235.687</v>
+        <v>24174.928</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>24873.128</v>
+        <v>24824.552</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>24867.671</v>
+        <v>24841.679</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>22803.77</v>
@@ -3238,7 +3238,7 @@
         <v>22803.77</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>24139.11</v>
+        <v>23513.79</v>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>看跌吞没</t>
+          <t>十字星</t>
         </is>
       </c>
       <c r="V4" s="2" t="n">

</xml_diff>

<commit_message>
auto stock scan 2026-10-29 14:49 UTC
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -3081,40 +3081,40 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
+        <v>11138.2</v>
+      </c>
+      <c r="D3" s="11" t="n">
         <v>11473.18</v>
       </c>
-      <c r="D3" s="11" t="n">
-        <v>11245.73</v>
-      </c>
       <c r="E3" s="11" t="n">
-        <v>11359.08</v>
+        <v>11379</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>11529.59</v>
+        <v>11379</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>11292.7</v>
-      </c>
-      <c r="H3" s="15" t="n">
-        <v>2.02</v>
+        <v>11135.97</v>
+      </c>
+      <c r="H3" s="12" t="n">
+        <v>-2.92</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>2.11</v>
+        <v>2.12</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>11456.887</v>
+        <v>11413.063</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>11622.675</v>
+        <v>11554.816</v>
       </c>
       <c r="L3" s="11" t="n">
-        <v>12646.137</v>
+        <v>12559.966</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>13303.794</v>
+        <v>13261.789</v>
       </c>
       <c r="N3" s="11" t="n">
-        <v>14305.939</v>
+        <v>14272.861</v>
       </c>
       <c r="O3" s="11" t="n">
         <v>11043.31</v>
@@ -3140,7 +3140,7 @@
       </c>
       <c r="U3" s="9" t="inlineStr">
         <is>
-          <t>看涨孕线</t>
+          <t>中阴线</t>
         </is>
       </c>
       <c r="V3" s="9" t="n">
@@ -3153,7 +3153,7 @@
       </c>
       <c r="X3" s="9" t="inlineStr">
         <is>
-          <t>跌破MA60 | 日内偏强</t>
+          <t>跌破MA60 | 日内偏弱</t>
         </is>
       </c>
     </row>
@@ -3169,52 +3169,52 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
+        <v>22958.65</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>23094.83</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>23041.32</v>
-      </c>
       <c r="E4" s="4" t="n">
-        <v>23083.99</v>
+        <v>23088.14</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>23157.4</v>
+        <v>23184.09</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>23023.04</v>
-      </c>
-      <c r="H4" s="14" t="n">
-        <v>0.23</v>
+        <v>22928.27</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>-0.59</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>0.58</v>
+        <v>1.11</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>23075.202</v>
+        <v>23079.996</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>23545.934</v>
+        <v>23410.382</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>24174.928</v>
+        <v>24117.975</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>24824.552</v>
+        <v>24776.314</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>24841.679</v>
+        <v>24811.116</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>22803.77</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>24524.63</v>
+        <v>24392.3</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>22803.77</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>23513.79</v>
+        <v>23313.92</v>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
@@ -3228,7 +3228,7 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>十字星</t>
+          <t>小阴线</t>
         </is>
       </c>
       <c r="V4" s="2" t="n">

</xml_diff>

<commit_message>
auto stock scan 2026-10-30 14:45 UTC
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -3153,40 +3153,40 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
+        <v>23294.42</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>22958.65</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>23094.83</v>
-      </c>
       <c r="E4" s="4" t="n">
-        <v>23088.14</v>
+        <v>23011.29</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>23184.09</v>
+        <v>23400.02</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>22928.27</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>-0.59</v>
+        <v>22947.96</v>
+      </c>
+      <c r="H4" s="16" t="n">
+        <v>1.46</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1.11</v>
+        <v>1.97</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>23079.996</v>
+        <v>23120.206</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>23410.382</v>
+        <v>23333.552</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>24117.975</v>
+        <v>24070.663</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>24776.314</v>
+        <v>24732.624</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>24811.116</v>
+        <v>24785.288</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>22803.77</v>
@@ -3195,10 +3195,10 @@
         <v>24392.3</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>22803.77</v>
+        <v>22928.27</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>23313.92</v>
+        <v>23400.02</v>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>小阴线</t>
+          <t>中阳线</t>
         </is>
       </c>
       <c r="V4" s="2" t="n">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>跌破MA60</t>
+          <t>跌破MA60 | 日内偏强</t>
         </is>
       </c>
     </row>
@@ -11933,7 +11933,7 @@
         <v>0.89</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>8.98</v>
+        <v>0.09</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
@@ -11944,7 +11944,7 @@
         <v>5.28</v>
       </c>
       <c r="P26" s="4" t="n">
-        <v>84.90000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="Q26" s="4" t="n">
         <v>0</v>
@@ -12268,7 +12268,7 @@
         <v>0.8</v>
       </c>
       <c r="M27" s="11" t="n">
-        <v>9.73</v>
+        <v>0.1</v>
       </c>
       <c r="N27" s="9" t="inlineStr">
         <is>
@@ -12279,7 +12279,7 @@
         <v>2.28</v>
       </c>
       <c r="P27" s="11" t="n">
-        <v>27.58</v>
+        <v>0.28</v>
       </c>
       <c r="Q27" s="11" t="n">
         <v>0</v>
@@ -12400,7 +12400,7 @@
         <v>-5</v>
       </c>
       <c r="AY27" s="11" t="n">
-        <v>3.25</v>
+        <v>3.24</v>
       </c>
       <c r="AZ27" s="9" t="n">
         <v>0</v>

</xml_diff>